<commit_message>
Perbaikan display detail AUX daily by agent, format upload file, penambahan chcker skip untuk error value pada kolom tanggal, persiapan form review WA
</commit_message>
<xml_diff>
--- a/files/Format_Upload_AUX_Daily.xlsx
+++ b/files/Format_Upload_AUX_Daily.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="682" uniqueCount="330">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="681" uniqueCount="330">
   <si>
     <t>Agent Name</t>
   </si>
@@ -489,466 +489,466 @@
     <t>:40:07</t>
   </si>
   <si>
+    <t xml:space="preserve"> 9:34:39</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 5:55:11</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 1:02:34</t>
+  </si>
+  <si>
+    <t>:26:38</t>
+  </si>
+  <si>
+    <t>:47:49</t>
+  </si>
+  <si>
+    <t>:40:09</t>
+  </si>
+  <si>
+    <t>:09:54</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 2:48:07</t>
+  </si>
+  <si>
+    <t>Intan</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 5:42:52</t>
+  </si>
+  <si>
+    <t>:10:37</t>
+  </si>
+  <si>
+    <t>:39:59</t>
+  </si>
+  <si>
+    <t>:01:41</t>
+  </si>
+  <si>
+    <t>:52:59</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 2:15:13</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 1:32:23</t>
+  </si>
+  <si>
+    <t>:10:00</t>
+  </si>
+  <si>
+    <t>Fahmi</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 9:15:32</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 5:24:21</t>
+  </si>
+  <si>
+    <t>:15:43</t>
+  </si>
+  <si>
+    <t>:37:27</t>
+  </si>
+  <si>
+    <t>:04:25</t>
+  </si>
+  <si>
+    <t>:36:14</t>
+  </si>
+  <si>
+    <t>:08:02</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 3:24:55</t>
+  </si>
+  <si>
+    <t>:17:35</t>
+  </si>
+  <si>
+    <t>Ayunda</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 9:20:58</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 5:20:27</t>
+  </si>
+  <si>
+    <t>:21:31</t>
+  </si>
+  <si>
+    <t>:24:41</t>
+  </si>
+  <si>
+    <t>:44:13</t>
+  </si>
+  <si>
+    <t>:39:36</t>
+  </si>
+  <si>
+    <t>:54:28</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 1:37:24</t>
+  </si>
+  <si>
+    <t>:38:34</t>
+  </si>
+  <si>
+    <t>Aguss</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 9:58:22</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 5:16:24</t>
+  </si>
+  <si>
+    <t>:50:44</t>
+  </si>
+  <si>
+    <t>:15:06</t>
+  </si>
+  <si>
+    <t>:21:12</t>
+  </si>
+  <si>
+    <t>:33:37</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 2:18:21</t>
+  </si>
+  <si>
+    <t>:57:24</t>
+  </si>
+  <si>
+    <t>Glorika</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 9:28:26</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 5:15:40</t>
+  </si>
+  <si>
+    <t>:54:12</t>
+  </si>
+  <si>
+    <t>:37:07</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 3:04:42</t>
+  </si>
+  <si>
+    <t>:29:39</t>
+  </si>
+  <si>
+    <t>Dina</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 9:46:02</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 4:54:00</t>
+  </si>
+  <si>
+    <t>:35:52</t>
+  </si>
+  <si>
+    <t>:57:22</t>
+  </si>
+  <si>
+    <t>:36:01</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 2:06:22</t>
+  </si>
+  <si>
+    <t>:38:23</t>
+  </si>
+  <si>
+    <t>Rina</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 4:50:03</t>
+  </si>
+  <si>
+    <t>:06:03</t>
+  </si>
+  <si>
+    <t>:13:22</t>
+  </si>
+  <si>
+    <t>:37:52</t>
+  </si>
+  <si>
+    <t>:17:44</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 3:30:22</t>
+  </si>
+  <si>
+    <t>:04:40</t>
+  </si>
+  <si>
+    <t>Arti</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 8:59:59</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 4:48:36</t>
+  </si>
+  <si>
+    <t>:33:35</t>
+  </si>
+  <si>
+    <t>:09:13</t>
+  </si>
+  <si>
+    <t>:38:17</t>
+  </si>
+  <si>
+    <t>:40:31</t>
+  </si>
+  <si>
+    <t>:19:44</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 1:05:58</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 1:10:44</t>
+  </si>
+  <si>
+    <t>:10:34</t>
+  </si>
+  <si>
+    <t>Rahma</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 9:55:12</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 4:41:22</t>
+  </si>
+  <si>
+    <t>:33:18</t>
+  </si>
+  <si>
+    <t>:42:50</t>
+  </si>
+  <si>
+    <t>:25:38</t>
+  </si>
+  <si>
+    <t>:39:37</t>
+  </si>
+  <si>
+    <t>:14:51</t>
+  </si>
+  <si>
+    <t>:44:22</t>
+  </si>
+  <si>
+    <t>:26:21</t>
+  </si>
+  <si>
+    <t>:54:25</t>
+  </si>
+  <si>
+    <t>Malik</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 4:40:51</t>
+  </si>
+  <si>
+    <t>:23:38</t>
+  </si>
+  <si>
+    <t>:32:01</t>
+  </si>
+  <si>
+    <t>:38:27</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 2:29:34</t>
+  </si>
+  <si>
+    <t>Tegar</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 9:53:51</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 4:33:49</t>
+  </si>
+  <si>
+    <t>:38:51</t>
+  </si>
+  <si>
+    <t>:21:29</t>
+  </si>
+  <si>
+    <t>:26:57</t>
+  </si>
+  <si>
+    <t>:43:12</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 1:28:56</t>
+  </si>
+  <si>
+    <t>:02:30</t>
+  </si>
+  <si>
+    <t>:51:54</t>
+  </si>
+  <si>
+    <t>Grace</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 9:22:57</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 3:49:05</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 1:22:29</t>
+  </si>
+  <si>
+    <t>:26:37</t>
+  </si>
+  <si>
+    <t>:01:18</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 1:00:47</t>
+  </si>
+  <si>
+    <t>:02:50</t>
+  </si>
+  <si>
+    <t>:15:35</t>
+  </si>
+  <si>
+    <t>Augita</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 6:25:02</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 3:47:08</t>
+  </si>
+  <si>
+    <t>:10:20</t>
+  </si>
+  <si>
+    <t>:06:58</t>
+  </si>
+  <si>
+    <t>:09:46</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 1:43:46</t>
+  </si>
+  <si>
+    <t>:01:10</t>
+  </si>
+  <si>
+    <t>:55:08</t>
+  </si>
+  <si>
+    <t>Zardi</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 3:42:23</t>
+  </si>
+  <si>
+    <t>:57:41</t>
+  </si>
+  <si>
+    <t>:44:09</t>
+  </si>
+  <si>
+    <t>:09:07</t>
+  </si>
+  <si>
+    <t>:40:27</t>
+  </si>
+  <si>
+    <t>:01:17</t>
+  </si>
+  <si>
+    <t>:08:01</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 1:00:31</t>
+  </si>
+  <si>
+    <t>Aliyah</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 6:12:59</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 3:02:33</t>
+  </si>
+  <si>
+    <t>:06:55</t>
+  </si>
+  <si>
+    <t>:22:44</t>
+  </si>
+  <si>
+    <t>:39:16</t>
+  </si>
+  <si>
+    <t>:02:13</t>
+  </si>
+  <si>
+    <t>:52:18</t>
+  </si>
+  <si>
+    <t>:00:52</t>
+  </si>
+  <si>
+    <t>:42:40</t>
+  </si>
+  <si>
+    <t>Aliahmad</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 1:23:14</t>
+  </si>
+  <si>
+    <t>:00:09</t>
+  </si>
+  <si>
+    <t>:40:04</t>
+  </si>
+  <si>
+    <t>:43:01</t>
+  </si>
+  <si>
+    <t>Nina</t>
+  </si>
+  <si>
+    <t>Logsheet ID</t>
+  </si>
+  <si>
+    <t>CMS Name</t>
+  </si>
+  <si>
+    <t>Extension</t>
+  </si>
+  <si>
     <t>Agam</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> 9:34:39</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> 5:55:11</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> 1:02:34</t>
-  </si>
-  <si>
-    <t>:26:38</t>
-  </si>
-  <si>
-    <t>:47:49</t>
-  </si>
-  <si>
-    <t>:40:09</t>
-  </si>
-  <si>
-    <t>:09:54</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> 2:48:07</t>
-  </si>
-  <si>
-    <t>Intan</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> 5:42:52</t>
-  </si>
-  <si>
-    <t>:10:37</t>
-  </si>
-  <si>
-    <t>:39:59</t>
-  </si>
-  <si>
-    <t>:01:41</t>
-  </si>
-  <si>
-    <t>:52:59</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> 2:15:13</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> 1:32:23</t>
-  </si>
-  <si>
-    <t>:10:00</t>
-  </si>
-  <si>
-    <t>Fahmi</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> 9:15:32</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> 5:24:21</t>
-  </si>
-  <si>
-    <t>:15:43</t>
-  </si>
-  <si>
-    <t>:37:27</t>
-  </si>
-  <si>
-    <t>:04:25</t>
-  </si>
-  <si>
-    <t>:36:14</t>
-  </si>
-  <si>
-    <t>:08:02</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> 3:24:55</t>
-  </si>
-  <si>
-    <t>:17:35</t>
-  </si>
-  <si>
-    <t>Ayunda</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> 9:20:58</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> 5:20:27</t>
-  </si>
-  <si>
-    <t>:21:31</t>
-  </si>
-  <si>
-    <t>:24:41</t>
-  </si>
-  <si>
-    <t>:44:13</t>
-  </si>
-  <si>
-    <t>:39:36</t>
-  </si>
-  <si>
-    <t>:54:28</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> 1:37:24</t>
-  </si>
-  <si>
-    <t>:38:34</t>
-  </si>
-  <si>
-    <t>Aguss</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> 9:58:22</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> 5:16:24</t>
-  </si>
-  <si>
-    <t>:50:44</t>
-  </si>
-  <si>
-    <t>:15:06</t>
-  </si>
-  <si>
-    <t>:21:12</t>
-  </si>
-  <si>
-    <t>:33:37</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> 2:18:21</t>
-  </si>
-  <si>
-    <t>:57:24</t>
-  </si>
-  <si>
-    <t>Glorika</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> 9:28:26</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> 5:15:40</t>
-  </si>
-  <si>
-    <t>:54:12</t>
-  </si>
-  <si>
-    <t>:37:07</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> 3:04:42</t>
-  </si>
-  <si>
-    <t>:29:39</t>
-  </si>
-  <si>
-    <t>Dina</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> 9:46:02</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> 4:54:00</t>
-  </si>
-  <si>
-    <t>:35:52</t>
-  </si>
-  <si>
-    <t>:57:22</t>
-  </si>
-  <si>
-    <t>:36:01</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> 2:06:22</t>
-  </si>
-  <si>
-    <t>:38:23</t>
-  </si>
-  <si>
-    <t>Rina</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> 4:50:03</t>
-  </si>
-  <si>
-    <t>:06:03</t>
-  </si>
-  <si>
-    <t>:13:22</t>
-  </si>
-  <si>
-    <t>:37:52</t>
-  </si>
-  <si>
-    <t>:17:44</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> 3:30:22</t>
-  </si>
-  <si>
-    <t>:04:40</t>
-  </si>
-  <si>
-    <t>Arti</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> 8:59:59</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> 4:48:36</t>
-  </si>
-  <si>
-    <t>:33:35</t>
-  </si>
-  <si>
-    <t>:09:13</t>
-  </si>
-  <si>
-    <t>:38:17</t>
-  </si>
-  <si>
-    <t>:40:31</t>
-  </si>
-  <si>
-    <t>:19:44</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> 1:05:58</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> 1:10:44</t>
-  </si>
-  <si>
-    <t>:10:34</t>
-  </si>
-  <si>
-    <t>Rahma</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> 9:55:12</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> 4:41:22</t>
-  </si>
-  <si>
-    <t>:33:18</t>
-  </si>
-  <si>
-    <t>:42:50</t>
-  </si>
-  <si>
-    <t>:25:38</t>
-  </si>
-  <si>
-    <t>:39:37</t>
-  </si>
-  <si>
-    <t>:14:51</t>
-  </si>
-  <si>
-    <t>:44:22</t>
-  </si>
-  <si>
-    <t>:26:21</t>
-  </si>
-  <si>
-    <t>:54:25</t>
-  </si>
-  <si>
-    <t>Malik</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> 4:40:51</t>
-  </si>
-  <si>
-    <t>:23:38</t>
-  </si>
-  <si>
-    <t>:32:01</t>
-  </si>
-  <si>
-    <t>:38:27</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> 2:29:34</t>
-  </si>
-  <si>
-    <t>Tegar</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> 9:53:51</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> 4:33:49</t>
-  </si>
-  <si>
-    <t>:38:51</t>
-  </si>
-  <si>
-    <t>:21:29</t>
-  </si>
-  <si>
-    <t>:26:57</t>
-  </si>
-  <si>
-    <t>:43:12</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> 1:28:56</t>
-  </si>
-  <si>
-    <t>:02:30</t>
-  </si>
-  <si>
-    <t>:51:54</t>
-  </si>
-  <si>
-    <t>Grace</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> 9:22:57</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> 3:49:05</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> 1:22:29</t>
-  </si>
-  <si>
-    <t>:26:37</t>
-  </si>
-  <si>
-    <t>:01:18</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> 1:00:47</t>
-  </si>
-  <si>
-    <t>:02:50</t>
-  </si>
-  <si>
-    <t>:15:35</t>
-  </si>
-  <si>
-    <t>Augita</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> 6:25:02</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> 3:47:08</t>
-  </si>
-  <si>
-    <t>:10:20</t>
-  </si>
-  <si>
-    <t>:06:58</t>
-  </si>
-  <si>
-    <t>:09:46</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> 1:43:46</t>
-  </si>
-  <si>
-    <t>:01:10</t>
-  </si>
-  <si>
-    <t>:55:08</t>
-  </si>
-  <si>
-    <t>Zardi</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> 3:42:23</t>
-  </si>
-  <si>
-    <t>:57:41</t>
-  </si>
-  <si>
-    <t>:44:09</t>
-  </si>
-  <si>
-    <t>:09:07</t>
-  </si>
-  <si>
-    <t>:40:27</t>
-  </si>
-  <si>
-    <t>:01:17</t>
-  </si>
-  <si>
-    <t>:08:01</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> 1:00:31</t>
-  </si>
-  <si>
-    <t>Aliyah</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> 6:12:59</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> 3:02:33</t>
-  </si>
-  <si>
-    <t>:06:55</t>
-  </si>
-  <si>
-    <t>:22:44</t>
-  </si>
-  <si>
-    <t>:39:16</t>
-  </si>
-  <si>
-    <t>:02:13</t>
-  </si>
-  <si>
-    <t>:52:18</t>
-  </si>
-  <si>
-    <t>:00:52</t>
-  </si>
-  <si>
-    <t>:42:40</t>
-  </si>
-  <si>
-    <t>Aliahmad</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> 1:23:14</t>
-  </si>
-  <si>
-    <t>:00:09</t>
-  </si>
-  <si>
-    <t>:40:04</t>
-  </si>
-  <si>
-    <t>:43:01</t>
-  </si>
-  <si>
-    <t>Nina</t>
-  </si>
-  <si>
-    <t>Logsheet ID</t>
-  </si>
-  <si>
-    <t>CMS Name</t>
-  </si>
-  <si>
-    <t>Extension</t>
   </si>
   <si>
     <t>Date</t>
@@ -1013,9 +1013,9 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="4">
+    <numFmt numFmtId="42" formatCode="_(&quot;$&quot;* #,##0_);_(&quot;$&quot;* \(#,##0\);_(&quot;$&quot;* &quot;-&quot;_);_(@_)"/>
     <numFmt numFmtId="176" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
     <numFmt numFmtId="44" formatCode="_(&quot;$&quot;* #,##0.00_);_(&quot;$&quot;* \(#,##0.00\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
-    <numFmt numFmtId="42" formatCode="_(&quot;$&quot;* #,##0_);_(&quot;$&quot;* \(#,##0\);_(&quot;$&quot;* &quot;-&quot;_);_(@_)"/>
     <numFmt numFmtId="177" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
   </numFmts>
   <fonts count="21">
@@ -1043,36 +1043,6 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="11"/>
-      <color theme="0"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FFFFFFFF"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FF3F3F3F"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
       <u/>
       <sz val="11"/>
       <color rgb="FF800080"/>
@@ -1090,18 +1060,24 @@
     </font>
     <font>
       <b/>
-      <sz val="11"/>
+      <sz val="13"/>
       <color theme="3"/>
       <name val="Calibri"/>
       <charset val="134"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <b/>
-      <sz val="15"/>
-      <color theme="3"/>
+      <sz val="11"/>
+      <color theme="1"/>
       <name val="Calibri"/>
-      <charset val="134"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="0"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -1113,33 +1089,11 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="11"/>
-      <color rgb="FF3F3F76"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
       <b/>
       <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="13"/>
       <color theme="3"/>
       <name val="Calibri"/>
       <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF9C0006"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -1158,10 +1112,56 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FF3F3F3F"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
       <sz val="11"/>
       <color rgb="FF9C6500"/>
       <name val="Calibri"/>
       <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF9C0006"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF3F3F76"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="15"/>
+      <color theme="3"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -1194,7 +1194,49 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFC6EFCE"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF2F2F2"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor theme="6" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFCC"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -1206,25 +1248,73 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="FFFFEB9C"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFC7CE"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFCC99"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="FFA5A5A5"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFF2F2F2"/>
+        <fgColor theme="5" tint="0.599993896298105"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="5"/>
+        <fgColor theme="8" tint="0.599993896298105"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.799981688894314"/>
+        <fgColor theme="6"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.799981688894314"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -1236,37 +1326,19 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFFCC99"/>
+        <fgColor theme="4" tint="0.399975585192419"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFFFFCC"/>
+        <fgColor theme="8" tint="0.399975585192419"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFC7CE"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFC6EFCE"/>
+        <fgColor theme="7" tint="0.399975585192419"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -1278,31 +1350,19 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.599993896298105"/>
+        <fgColor theme="7"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.599993896298105"/>
+        <fgColor theme="8" tint="0.799981688894314"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.799981688894314"/>
+        <fgColor theme="9" tint="0.599993896298105"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -1314,67 +1374,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFEB9C"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor theme="9"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.599993896298105"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -1397,32 +1397,11 @@
       <diagonal/>
     </border>
     <border>
-      <left style="double">
-        <color rgb="FF3F3F3F"/>
-      </left>
-      <right style="double">
-        <color rgb="FF3F3F3F"/>
-      </right>
-      <top style="double">
-        <color rgb="FF3F3F3F"/>
-      </top>
-      <bottom style="double">
-        <color rgb="FF3F3F3F"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF3F3F3F"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF3F3F3F"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF3F3F3F"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF3F3F3F"/>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color theme="4"/>
       </bottom>
       <diagonal/>
     </border>
@@ -1432,15 +1411,6 @@
       <top/>
       <bottom style="medium">
         <color theme="4" tint="0.499984740745262"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="medium">
-        <color theme="4"/>
       </bottom>
       <diagonal/>
     </border>
@@ -1475,6 +1445,21 @@
       <diagonal/>
     </border>
     <border>
+      <left style="thin">
+        <color rgb="FF3F3F3F"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF3F3F3F"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF3F3F3F"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF3F3F3F"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
       <left/>
       <right/>
       <top style="thin">
@@ -1482,6 +1467,21 @@
       </top>
       <bottom style="double">
         <color theme="4"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="double">
+        <color rgb="FF3F3F3F"/>
+      </left>
+      <right style="double">
+        <color rgb="FF3F3F3F"/>
+      </right>
+      <top style="double">
+        <color rgb="FF3F3F3F"/>
+      </top>
+      <bottom style="double">
+        <color rgb="FF3F3F3F"/>
       </bottom>
       <diagonal/>
     </border>
@@ -1497,121 +1497,121 @@
   </borders>
   <cellStyleXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="7" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="6" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="7" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="7" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="6" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="6" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="7" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="7" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="6" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="7" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="20" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="6" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="7" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="7" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="6" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="6" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="6" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="6" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="7" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="14" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="7" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="15" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="6" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="6" borderId="3" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="12" fillId="7" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="44" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="7" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="5" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="10" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="16" fillId="14" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="6" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="11" fillId="7" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="10" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="5" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="177" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="42" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
@@ -1620,19 +1620,19 @@
     <xf numFmtId="0" fontId="19" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="5" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="176" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="2" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="17" fillId="16" borderId="8" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="7" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
@@ -1990,15 +1990,15 @@
   <sheetPr>
     <tabColor theme="7" tint="0.4"/>
   </sheetPr>
-  <dimension ref="A1:AG36"/>
+  <dimension ref="A1:AI36"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
   <cols>
-    <col min="31" max="31" width="3.25" style="4" customWidth="1"/>
-    <col min="32" max="32" width="9" style="5"/>
-    <col min="33" max="33" width="11.125" style="5" customWidth="1"/>
+    <col min="31" max="33" width="1.75" style="4" customWidth="1"/>
+    <col min="34" max="34" width="9" style="5"/>
+    <col min="35" max="35" width="11.125" style="5" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:33">
+    <row r="1" spans="1:35">
       <c r="A1" s="6" t="s">
         <v>0</v>
       </c>
@@ -2059,14 +2059,14 @@
       <c r="AB1" s="6"/>
       <c r="AC1" s="6"/>
       <c r="AD1" s="6"/>
-      <c r="AF1" s="5" t="s">
+      <c r="AH1" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="AG1" s="5" t="s">
+      <c r="AI1" s="5" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="2" spans="1:33">
+    <row r="2" spans="1:35">
       <c r="A2" s="6" t="s">
         <v>17</v>
       </c>
@@ -2157,14 +2157,14 @@
       <c r="AD2" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="AF2" s="9">
-        <v>46171</v>
-      </c>
-      <c r="AG2" s="5">
+      <c r="AH2" s="9">
+        <v>46154</v>
+      </c>
+      <c r="AI2" s="5">
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:33">
+    <row r="3" spans="1:35">
       <c r="A3" s="6" t="s">
         <v>20</v>
       </c>
@@ -2255,14 +2255,14 @@
       <c r="AD3" s="6">
         <v>36969</v>
       </c>
-      <c r="AF3" s="9">
-        <v>46171</v>
-      </c>
-      <c r="AG3" s="5">
+      <c r="AH3" s="9">
+        <v>46154</v>
+      </c>
+      <c r="AI3" s="5">
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:33">
+    <row r="4" spans="1:35">
       <c r="A4" s="6" t="s">
         <v>27</v>
       </c>
@@ -2353,14 +2353,14 @@
       <c r="AD4" s="6">
         <v>34799</v>
       </c>
-      <c r="AF4" s="9">
-        <v>46171</v>
-      </c>
-      <c r="AG4" s="5">
+      <c r="AH4" s="9">
+        <v>46154</v>
+      </c>
+      <c r="AI4" s="5">
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="1:33">
+    <row r="5" spans="1:35">
       <c r="A5" s="6" t="s">
         <v>34</v>
       </c>
@@ -2451,14 +2451,14 @@
       <c r="AD5" s="6">
         <v>34785</v>
       </c>
-      <c r="AF5" s="9">
-        <v>46171</v>
-      </c>
-      <c r="AG5" s="5">
+      <c r="AH5" s="9">
+        <v>46154</v>
+      </c>
+      <c r="AI5" s="5">
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="1:33">
+    <row r="6" spans="1:35">
       <c r="A6" s="6" t="s">
         <v>40</v>
       </c>
@@ -2549,14 +2549,14 @@
       <c r="AD6" s="6">
         <v>34060</v>
       </c>
-      <c r="AF6" s="9">
-        <v>46171</v>
-      </c>
-      <c r="AG6" s="5">
+      <c r="AH6" s="9">
+        <v>46154</v>
+      </c>
+      <c r="AI6" s="5">
         <v>1</v>
       </c>
     </row>
-    <row r="7" spans="1:33">
+    <row r="7" spans="1:35">
       <c r="A7" s="6" t="s">
         <v>47</v>
       </c>
@@ -2647,14 +2647,14 @@
       <c r="AD7" s="6">
         <v>33788</v>
       </c>
-      <c r="AF7" s="9">
-        <v>46171</v>
-      </c>
-      <c r="AG7" s="5">
+      <c r="AH7" s="9">
+        <v>46154</v>
+      </c>
+      <c r="AI7" s="5">
         <v>1</v>
       </c>
     </row>
-    <row r="8" spans="1:33">
+    <row r="8" spans="1:35">
       <c r="A8" s="6" t="s">
         <v>55</v>
       </c>
@@ -2745,14 +2745,14 @@
       <c r="AD8" s="6">
         <v>33154</v>
       </c>
-      <c r="AF8" s="9">
-        <v>46171</v>
-      </c>
-      <c r="AG8" s="5">
+      <c r="AH8" s="9">
+        <v>46154</v>
+      </c>
+      <c r="AI8" s="5">
         <v>1</v>
       </c>
     </row>
-    <row r="9" spans="1:33">
+    <row r="9" spans="1:35">
       <c r="A9" s="6" t="s">
         <v>64</v>
       </c>
@@ -2843,14 +2843,14 @@
       <c r="AD9" s="6">
         <v>33057</v>
       </c>
-      <c r="AF9" s="9">
-        <v>46171</v>
-      </c>
-      <c r="AG9" s="5">
+      <c r="AH9" s="9">
+        <v>46154</v>
+      </c>
+      <c r="AI9" s="5">
         <v>1</v>
       </c>
     </row>
-    <row r="10" spans="1:33">
+    <row r="10" spans="1:35">
       <c r="A10" s="6" t="s">
         <v>71</v>
       </c>
@@ -2941,14 +2941,14 @@
       <c r="AD10" s="6">
         <v>32964</v>
       </c>
-      <c r="AF10" s="9">
-        <v>46171</v>
-      </c>
-      <c r="AG10" s="5">
+      <c r="AH10" s="9">
+        <v>46154</v>
+      </c>
+      <c r="AI10" s="5">
         <v>1</v>
       </c>
     </row>
-    <row r="11" spans="1:33">
+    <row r="11" spans="1:35">
       <c r="A11" s="6" t="s">
         <v>81</v>
       </c>
@@ -3039,14 +3039,14 @@
       <c r="AD11" s="6">
         <v>28830</v>
       </c>
-      <c r="AF11" s="9">
-        <v>46171</v>
-      </c>
-      <c r="AG11" s="5">
+      <c r="AH11" s="9">
+        <v>46154</v>
+      </c>
+      <c r="AI11" s="5">
         <v>1</v>
       </c>
     </row>
-    <row r="12" spans="1:33">
+    <row r="12" spans="1:35">
       <c r="A12" s="6" t="s">
         <v>92</v>
       </c>
@@ -3137,14 +3137,14 @@
       <c r="AD12" s="6">
         <v>28350</v>
       </c>
-      <c r="AF12" s="9">
-        <v>46171</v>
-      </c>
-      <c r="AG12" s="5">
+      <c r="AH12" s="9">
+        <v>46154</v>
+      </c>
+      <c r="AI12" s="5">
         <v>1</v>
       </c>
     </row>
-    <row r="13" spans="1:33">
+    <row r="13" spans="1:35">
       <c r="A13" s="6" t="s">
         <v>102</v>
       </c>
@@ -3235,14 +3235,14 @@
       <c r="AD13" s="6">
         <v>27007</v>
       </c>
-      <c r="AF13" s="9">
-        <v>46171</v>
-      </c>
-      <c r="AG13" s="5">
+      <c r="AH13" s="9">
+        <v>46154</v>
+      </c>
+      <c r="AI13" s="5">
         <v>1</v>
       </c>
     </row>
-    <row r="14" spans="1:33">
+    <row r="14" spans="1:35">
       <c r="A14" s="6" t="s">
         <v>113</v>
       </c>
@@ -3333,14 +3333,14 @@
       <c r="AD14" s="6">
         <v>26285</v>
       </c>
-      <c r="AF14" s="9">
-        <v>46171</v>
-      </c>
-      <c r="AG14" s="5">
+      <c r="AH14" s="9">
+        <v>46154</v>
+      </c>
+      <c r="AI14" s="5">
         <v>1</v>
       </c>
     </row>
-    <row r="15" spans="1:33">
+    <row r="15" spans="1:35">
       <c r="A15" s="6" t="s">
         <v>122</v>
       </c>
@@ -3431,14 +3431,14 @@
       <c r="AD15" s="6">
         <v>23785</v>
       </c>
-      <c r="AF15" s="9">
-        <v>46171</v>
-      </c>
-      <c r="AG15" s="5">
+      <c r="AH15" s="9">
+        <v>46154</v>
+      </c>
+      <c r="AI15" s="5">
         <v>1</v>
       </c>
     </row>
-    <row r="16" spans="1:33">
+    <row r="16" spans="1:35">
       <c r="A16" s="6" t="s">
         <v>131</v>
       </c>
@@ -3529,14 +3529,14 @@
       <c r="AD16" s="6">
         <v>21995</v>
       </c>
-      <c r="AF16" s="9">
-        <v>46171</v>
-      </c>
-      <c r="AG16" s="5">
+      <c r="AH16" s="9">
+        <v>46154</v>
+      </c>
+      <c r="AI16" s="5">
         <v>1</v>
       </c>
     </row>
-    <row r="17" spans="1:33">
+    <row r="17" spans="1:35">
       <c r="A17" s="6" t="s">
         <v>139</v>
       </c>
@@ -3627,14 +3627,14 @@
       <c r="AD17" s="6">
         <v>21879</v>
       </c>
-      <c r="AF17" s="9">
-        <v>46171</v>
-      </c>
-      <c r="AG17" s="5">
+      <c r="AH17" s="9">
+        <v>46154</v>
+      </c>
+      <c r="AI17" s="5">
         <v>1</v>
       </c>
     </row>
-    <row r="18" spans="1:33">
+    <row r="18" spans="1:35">
       <c r="A18" s="6" t="s">
         <v>147</v>
       </c>
@@ -3725,17 +3725,15 @@
       <c r="AD18" s="6">
         <v>21467</v>
       </c>
-      <c r="AF18" s="9">
-        <v>46171</v>
-      </c>
-      <c r="AG18" s="5">
+      <c r="AH18" s="9">
+        <v>46154</v>
+      </c>
+      <c r="AI18" s="5">
         <v>1</v>
       </c>
     </row>
-    <row r="19" spans="1:33">
-      <c r="A19" s="6" t="s">
-        <v>157</v>
-      </c>
+    <row r="19" spans="1:35">
+      <c r="A19" s="6"/>
       <c r="B19" s="6">
         <v>1648</v>
       </c>
@@ -3743,37 +3741,37 @@
         <v>34479</v>
       </c>
       <c r="D19" s="6" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="E19" s="6">
         <v>21311</v>
       </c>
       <c r="F19" s="6" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="G19" s="6">
         <v>3754</v>
       </c>
       <c r="H19" s="6" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="I19" s="6">
         <v>1598</v>
       </c>
       <c r="J19" s="6" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="K19" s="6">
         <v>2869</v>
       </c>
       <c r="L19" s="6" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="M19" s="6">
         <v>2409</v>
       </c>
       <c r="N19" s="6" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="O19" s="6">
         <v>0</v>
@@ -3785,13 +3783,13 @@
         <v>594</v>
       </c>
       <c r="R19" s="6" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="S19" s="6">
         <v>10087</v>
       </c>
       <c r="T19" s="6" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="U19" s="6">
         <v>0</v>
@@ -3823,16 +3821,16 @@
       <c r="AD19" s="6">
         <v>21311</v>
       </c>
-      <c r="AF19" s="9">
-        <v>46171</v>
-      </c>
-      <c r="AG19" s="5">
+      <c r="AH19" s="9">
+        <v>46154</v>
+      </c>
+      <c r="AI19" s="5">
         <v>1</v>
       </c>
     </row>
-    <row r="20" spans="1:33">
+    <row r="20" spans="1:35">
       <c r="A20" s="6" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="B20" s="6">
         <v>1651</v>
@@ -3847,31 +3845,31 @@
         <v>20572</v>
       </c>
       <c r="F20" s="6" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="G20" s="6">
         <v>637</v>
       </c>
       <c r="H20" s="6" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="I20" s="6">
         <v>2399</v>
       </c>
       <c r="J20" s="6" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="K20" s="6">
         <v>101</v>
       </c>
       <c r="L20" s="6" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="M20" s="6">
         <v>3179</v>
       </c>
       <c r="N20" s="6" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="O20" s="6">
         <v>0</v>
@@ -3883,13 +3881,13 @@
         <v>8113</v>
       </c>
       <c r="R20" s="6" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="S20" s="6">
         <v>5543</v>
       </c>
       <c r="T20" s="6" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="U20" s="6">
         <v>0</v>
@@ -3907,7 +3905,7 @@
         <v>600</v>
       </c>
       <c r="Z20" s="6" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="AA20" s="6">
         <v>0</v>
@@ -3921,16 +3919,16 @@
       <c r="AD20" s="6">
         <v>20572</v>
       </c>
-      <c r="AF20" s="9">
-        <v>46171</v>
-      </c>
-      <c r="AG20" s="5">
+      <c r="AH20" s="9">
+        <v>46154</v>
+      </c>
+      <c r="AI20" s="5">
         <v>1</v>
       </c>
     </row>
-    <row r="21" spans="1:33">
+    <row r="21" spans="1:35">
       <c r="A21" s="6" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="B21" s="6">
         <v>1628</v>
@@ -3939,37 +3937,37 @@
         <v>33332</v>
       </c>
       <c r="D21" s="6" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="E21" s="6">
         <v>19461</v>
       </c>
       <c r="F21" s="6" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="G21" s="6">
         <v>943</v>
       </c>
       <c r="H21" s="6" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="I21" s="6">
         <v>2247</v>
       </c>
       <c r="J21" s="6" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="K21" s="6">
         <v>265</v>
       </c>
       <c r="L21" s="6" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="M21" s="6">
         <v>2174</v>
       </c>
       <c r="N21" s="6" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="O21" s="6">
         <v>0</v>
@@ -3981,13 +3979,13 @@
         <v>482</v>
       </c>
       <c r="R21" s="6" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="S21" s="6">
         <v>12295</v>
       </c>
       <c r="T21" s="6" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="U21" s="6">
         <v>0</v>
@@ -4005,7 +4003,7 @@
         <v>1055</v>
       </c>
       <c r="Z21" s="6" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="AA21" s="6">
         <v>0</v>
@@ -4019,16 +4017,16 @@
       <c r="AD21" s="6">
         <v>19461</v>
       </c>
-      <c r="AF21" s="9">
-        <v>46171</v>
-      </c>
-      <c r="AG21" s="5">
+      <c r="AH21" s="9">
+        <v>46154</v>
+      </c>
+      <c r="AI21" s="5">
         <v>1</v>
       </c>
     </row>
-    <row r="22" spans="1:33">
+    <row r="22" spans="1:35">
       <c r="A22" s="6" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="B22" s="6">
         <v>1635</v>
@@ -4037,37 +4035,37 @@
         <v>33658</v>
       </c>
       <c r="D22" s="6" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="E22" s="6">
         <v>19227</v>
       </c>
       <c r="F22" s="6" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="G22" s="6">
         <v>1291</v>
       </c>
       <c r="H22" s="6" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="I22" s="6">
         <v>1481</v>
       </c>
       <c r="J22" s="6" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="K22" s="6">
         <v>2653</v>
       </c>
       <c r="L22" s="6" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="M22" s="6">
         <v>2376</v>
       </c>
       <c r="N22" s="6" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="O22" s="6">
         <v>0</v>
@@ -4079,13 +4077,13 @@
         <v>3268</v>
       </c>
       <c r="R22" s="6" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="S22" s="6">
         <v>5844</v>
       </c>
       <c r="T22" s="6" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="U22" s="6">
         <v>0</v>
@@ -4103,7 +4101,7 @@
         <v>2314</v>
       </c>
       <c r="Z22" s="6" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="AA22" s="6">
         <v>0</v>
@@ -4117,16 +4115,16 @@
       <c r="AD22" s="6">
         <v>19227</v>
       </c>
-      <c r="AF22" s="9">
-        <v>46171</v>
-      </c>
-      <c r="AG22" s="5">
+      <c r="AH22" s="9">
+        <v>46154</v>
+      </c>
+      <c r="AI22" s="5">
         <v>1</v>
       </c>
     </row>
-    <row r="23" spans="1:33">
+    <row r="23" spans="1:35">
       <c r="A23" s="6" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="B23" s="6">
         <v>1636</v>
@@ -4135,37 +4133,37 @@
         <v>35902</v>
       </c>
       <c r="D23" s="6" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="E23" s="6">
         <v>18984</v>
       </c>
       <c r="F23" s="6" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="G23" s="6">
         <v>3044</v>
       </c>
       <c r="H23" s="6" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="I23" s="6">
         <v>906</v>
       </c>
       <c r="J23" s="6" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="K23" s="6">
         <v>1272</v>
       </c>
       <c r="L23" s="6" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="M23" s="6">
         <v>2017</v>
       </c>
       <c r="N23" s="6" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="O23" s="6">
         <v>0</v>
@@ -4183,7 +4181,7 @@
         <v>8301</v>
       </c>
       <c r="T23" s="6" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="U23" s="6">
         <v>0</v>
@@ -4201,7 +4199,7 @@
         <v>3444</v>
       </c>
       <c r="Z23" s="6" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="AA23" s="6">
         <v>0</v>
@@ -4215,16 +4213,16 @@
       <c r="AD23" s="6">
         <v>18984</v>
       </c>
-      <c r="AF23" s="9">
-        <v>46171</v>
-      </c>
-      <c r="AG23" s="5">
+      <c r="AH23" s="9">
+        <v>46154</v>
+      </c>
+      <c r="AI23" s="5">
         <v>1</v>
       </c>
     </row>
-    <row r="24" spans="1:33">
+    <row r="24" spans="1:35">
       <c r="A24" s="6" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="B24" s="6">
         <v>1642</v>
@@ -4233,19 +4231,19 @@
         <v>34106</v>
       </c>
       <c r="D24" s="6" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="E24" s="6">
         <v>18940</v>
       </c>
       <c r="F24" s="6" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="G24" s="6">
         <v>3252</v>
       </c>
       <c r="H24" s="6" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="I24" s="6">
         <v>0</v>
@@ -4257,13 +4255,13 @@
         <v>600</v>
       </c>
       <c r="L24" s="6" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="M24" s="6">
         <v>2227</v>
       </c>
       <c r="N24" s="6" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="O24" s="6">
         <v>0</v>
@@ -4281,7 +4279,7 @@
         <v>11082</v>
       </c>
       <c r="T24" s="6" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="U24" s="6">
         <v>0</v>
@@ -4299,7 +4297,7 @@
         <v>1779</v>
       </c>
       <c r="Z24" s="6" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="AA24" s="6">
         <v>0</v>
@@ -4313,16 +4311,16 @@
       <c r="AD24" s="6">
         <v>18940</v>
       </c>
-      <c r="AF24" s="9">
-        <v>46171</v>
-      </c>
-      <c r="AG24" s="5">
+      <c r="AH24" s="9">
+        <v>46154</v>
+      </c>
+      <c r="AI24" s="5">
         <v>1</v>
       </c>
     </row>
-    <row r="25" spans="1:33">
+    <row r="25" spans="1:35">
       <c r="A25" s="6" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="B25" s="6">
         <v>1624</v>
@@ -4331,19 +4329,19 @@
         <v>35162</v>
       </c>
       <c r="D25" s="6" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="E25" s="6">
         <v>17640</v>
       </c>
       <c r="F25" s="6" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="G25" s="6">
         <v>2152</v>
       </c>
       <c r="H25" s="6" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="I25" s="6">
         <v>0</v>
@@ -4355,13 +4353,13 @@
         <v>3442</v>
       </c>
       <c r="L25" s="6" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="M25" s="6">
         <v>2161</v>
       </c>
       <c r="N25" s="6" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="O25" s="6">
         <v>0</v>
@@ -4379,7 +4377,7 @@
         <v>7582</v>
       </c>
       <c r="T25" s="6" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="U25" s="6">
         <v>0</v>
@@ -4397,7 +4395,7 @@
         <v>2303</v>
       </c>
       <c r="Z25" s="6" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="AA25" s="6">
         <v>0</v>
@@ -4411,16 +4409,16 @@
       <c r="AD25" s="6">
         <v>17640</v>
       </c>
-      <c r="AF25" s="9">
-        <v>46171</v>
-      </c>
-      <c r="AG25" s="5">
+      <c r="AH25" s="9">
+        <v>46154</v>
+      </c>
+      <c r="AI25" s="5">
         <v>1</v>
       </c>
     </row>
-    <row r="26" spans="1:33">
+    <row r="26" spans="1:35">
       <c r="A26" s="6" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="B26" s="6">
         <v>1653</v>
@@ -4435,13 +4433,13 @@
         <v>17403</v>
       </c>
       <c r="F26" s="6" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="G26" s="6">
         <v>363</v>
       </c>
       <c r="H26" s="6" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="I26" s="6">
         <v>0</v>
@@ -4453,13 +4451,13 @@
         <v>802</v>
       </c>
       <c r="L26" s="6" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="M26" s="6">
         <v>2272</v>
       </c>
       <c r="N26" s="6" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="O26" s="6">
         <v>0</v>
@@ -4471,13 +4469,13 @@
         <v>1064</v>
       </c>
       <c r="R26" s="6" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="S26" s="6">
         <v>12622</v>
       </c>
       <c r="T26" s="6" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="U26" s="6">
         <v>0</v>
@@ -4495,7 +4493,7 @@
         <v>280</v>
       </c>
       <c r="Z26" s="6" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="AA26" s="6">
         <v>0</v>
@@ -4509,16 +4507,16 @@
       <c r="AD26" s="6">
         <v>17403</v>
       </c>
-      <c r="AF26" s="9">
-        <v>46171</v>
-      </c>
-      <c r="AG26" s="5">
+      <c r="AH26" s="9">
+        <v>46154</v>
+      </c>
+      <c r="AI26" s="5">
         <v>1</v>
       </c>
     </row>
-    <row r="27" spans="1:33">
+    <row r="27" spans="1:35">
       <c r="A27" s="6" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="B27" s="6">
         <v>1622</v>
@@ -4527,37 +4525,37 @@
         <v>32399</v>
       </c>
       <c r="D27" s="6" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="E27" s="6">
         <v>17316</v>
       </c>
       <c r="F27" s="6" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="G27" s="6">
         <v>2015</v>
       </c>
       <c r="H27" s="6" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="I27" s="6">
         <v>553</v>
       </c>
       <c r="J27" s="6" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="K27" s="6">
         <v>2297</v>
       </c>
       <c r="L27" s="6" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="M27" s="6">
         <v>2431</v>
       </c>
       <c r="N27" s="6" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="O27" s="6">
         <v>0</v>
@@ -4569,13 +4567,13 @@
         <v>1184</v>
       </c>
       <c r="R27" s="6" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="S27" s="6">
         <v>3958</v>
       </c>
       <c r="T27" s="6" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="U27" s="6">
         <v>0</v>
@@ -4587,13 +4585,13 @@
         <v>4244</v>
       </c>
       <c r="X27" s="6" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="Y27" s="6">
         <v>634</v>
       </c>
       <c r="Z27" s="6" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="AA27" s="6">
         <v>0</v>
@@ -4607,16 +4605,16 @@
       <c r="AD27" s="6">
         <v>17316</v>
       </c>
-      <c r="AF27" s="9">
-        <v>46171</v>
-      </c>
-      <c r="AG27" s="5">
+      <c r="AH27" s="9">
+        <v>46154</v>
+      </c>
+      <c r="AI27" s="5">
         <v>1</v>
       </c>
     </row>
-    <row r="28" spans="1:33">
+    <row r="28" spans="1:35">
       <c r="A28" s="6" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="B28" s="6">
         <v>1630</v>
@@ -4625,37 +4623,37 @@
         <v>35712</v>
       </c>
       <c r="D28" s="6" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="E28" s="6">
         <v>16882</v>
       </c>
       <c r="F28" s="6" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="G28" s="6">
         <v>1998</v>
       </c>
       <c r="H28" s="6" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="I28" s="6">
         <v>2570</v>
       </c>
       <c r="J28" s="6" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="K28" s="6">
         <v>1538</v>
       </c>
       <c r="L28" s="6" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="M28" s="6">
         <v>2377</v>
       </c>
       <c r="N28" s="6" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="O28" s="6">
         <v>0</v>
@@ -4667,13 +4665,13 @@
         <v>891</v>
       </c>
       <c r="R28" s="6" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="S28" s="6">
         <v>2662</v>
       </c>
       <c r="T28" s="6" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="U28" s="6">
         <v>0</v>
@@ -4685,13 +4683,13 @@
         <v>1581</v>
       </c>
       <c r="X28" s="6" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="Y28" s="6">
         <v>3265</v>
       </c>
       <c r="Z28" s="6" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="AA28" s="6">
         <v>0</v>
@@ -4705,16 +4703,16 @@
       <c r="AD28" s="6">
         <v>16882</v>
       </c>
-      <c r="AF28" s="9">
-        <v>46171</v>
-      </c>
-      <c r="AG28" s="5">
+      <c r="AH28" s="9">
+        <v>46154</v>
+      </c>
+      <c r="AI28" s="5">
         <v>1</v>
       </c>
     </row>
-    <row r="29" spans="1:33">
+    <row r="29" spans="1:35">
       <c r="A29" s="6" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="B29" s="6">
         <v>1632</v>
@@ -4729,13 +4727,13 @@
         <v>16851</v>
       </c>
       <c r="F29" s="6" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="G29" s="6">
         <v>1418</v>
       </c>
       <c r="H29" s="6" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="I29" s="6">
         <v>2231</v>
@@ -4747,13 +4745,13 @@
         <v>1921</v>
       </c>
       <c r="L29" s="6" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="M29" s="6">
         <v>2307</v>
       </c>
       <c r="N29" s="6" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="O29" s="6">
         <v>0</v>
@@ -4771,7 +4769,7 @@
         <v>8974</v>
       </c>
       <c r="T29" s="6" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
       <c r="U29" s="6">
         <v>0</v>
@@ -4803,16 +4801,16 @@
       <c r="AD29" s="6">
         <v>16851</v>
       </c>
-      <c r="AF29" s="9">
-        <v>46171</v>
-      </c>
-      <c r="AG29" s="5">
+      <c r="AH29" s="9">
+        <v>46154</v>
+      </c>
+      <c r="AI29" s="5">
         <v>1</v>
       </c>
     </row>
-    <row r="30" spans="1:33">
+    <row r="30" spans="1:35">
       <c r="A30" s="6" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="B30" s="6">
         <v>1641</v>
@@ -4821,37 +4819,37 @@
         <v>35631</v>
       </c>
       <c r="D30" s="6" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="E30" s="6">
         <v>16429</v>
       </c>
       <c r="F30" s="6" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="G30" s="6">
         <v>2331</v>
       </c>
       <c r="H30" s="6" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="I30" s="6">
         <v>1289</v>
       </c>
       <c r="J30" s="6" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="K30" s="6">
         <v>1617</v>
       </c>
       <c r="L30" s="6" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="M30" s="6">
         <v>2592</v>
       </c>
       <c r="N30" s="6" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="O30" s="6">
         <v>0</v>
@@ -4869,7 +4867,7 @@
         <v>5336</v>
       </c>
       <c r="T30" s="6" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="U30" s="6">
         <v>0</v>
@@ -4881,13 +4879,13 @@
         <v>150</v>
       </c>
       <c r="X30" s="6" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="Y30" s="6">
         <v>3114</v>
       </c>
       <c r="Z30" s="6" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="AA30" s="6">
         <v>0</v>
@@ -4901,16 +4899,16 @@
       <c r="AD30" s="6">
         <v>16429</v>
       </c>
-      <c r="AF30" s="9">
-        <v>46171</v>
-      </c>
-      <c r="AG30" s="5">
+      <c r="AH30" s="9">
+        <v>46154</v>
+      </c>
+      <c r="AI30" s="5">
         <v>1</v>
       </c>
     </row>
-    <row r="31" spans="1:33">
+    <row r="31" spans="1:35">
       <c r="A31" s="6" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="B31" s="6">
         <v>1647</v>
@@ -4919,19 +4917,19 @@
         <v>33777</v>
       </c>
       <c r="D31" s="6" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="E31" s="6">
         <v>13745</v>
       </c>
       <c r="F31" s="6" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="G31" s="6">
         <v>4949</v>
       </c>
       <c r="H31" s="6" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="I31" s="6">
         <v>0</v>
@@ -4943,7 +4941,7 @@
         <v>1597</v>
       </c>
       <c r="L31" s="6" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="M31" s="6">
         <v>2369</v>
@@ -4961,13 +4959,13 @@
         <v>78</v>
       </c>
       <c r="R31" s="6" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
       <c r="S31" s="6">
         <v>3647</v>
       </c>
       <c r="T31" s="6" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="U31" s="6">
         <v>0</v>
@@ -4979,13 +4977,13 @@
         <v>170</v>
       </c>
       <c r="X31" s="6" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="Y31" s="6">
         <v>935</v>
       </c>
       <c r="Z31" s="6" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="AA31" s="6">
         <v>0</v>
@@ -4999,16 +4997,16 @@
       <c r="AD31" s="6">
         <v>13745</v>
       </c>
-      <c r="AF31" s="9">
-        <v>46171</v>
-      </c>
-      <c r="AG31" s="5">
+      <c r="AH31" s="9">
+        <v>46154</v>
+      </c>
+      <c r="AI31" s="5">
         <v>1</v>
       </c>
     </row>
-    <row r="32" spans="1:33">
+    <row r="32" spans="1:35">
       <c r="A32" s="6" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="B32" s="6">
         <v>1652</v>
@@ -5017,19 +5015,19 @@
         <v>23102</v>
       </c>
       <c r="D32" s="6" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="E32" s="6">
         <v>13628</v>
       </c>
       <c r="F32" s="6" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="G32" s="6">
         <v>620</v>
       </c>
       <c r="H32" s="6" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="I32" s="6">
         <v>0</v>
@@ -5041,7 +5039,7 @@
         <v>418</v>
       </c>
       <c r="L32" s="6" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="M32" s="6">
         <v>2400</v>
@@ -5059,13 +5057,13 @@
         <v>586</v>
       </c>
       <c r="R32" s="6" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="S32" s="6">
         <v>6226</v>
       </c>
       <c r="T32" s="6" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="U32" s="6">
         <v>0</v>
@@ -5077,13 +5075,13 @@
         <v>70</v>
       </c>
       <c r="X32" s="6" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="Y32" s="6">
         <v>3308</v>
       </c>
       <c r="Z32" s="6" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
       <c r="AA32" s="6">
         <v>0</v>
@@ -5097,16 +5095,16 @@
       <c r="AD32" s="6">
         <v>13628</v>
       </c>
-      <c r="AF32" s="9">
-        <v>46171</v>
-      </c>
-      <c r="AG32" s="5">
+      <c r="AH32" s="9">
+        <v>46154</v>
+      </c>
+      <c r="AI32" s="5">
         <v>1</v>
       </c>
     </row>
-    <row r="33" spans="1:33">
+    <row r="33" spans="1:35">
       <c r="A33" s="6" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
       <c r="B33" s="6">
         <v>1621</v>
@@ -5121,31 +5119,31 @@
         <v>13343</v>
       </c>
       <c r="F33" s="6" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="G33" s="6">
         <v>3461</v>
       </c>
       <c r="H33" s="6" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
       <c r="I33" s="6">
         <v>2649</v>
       </c>
       <c r="J33" s="6" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="K33" s="6">
         <v>547</v>
       </c>
       <c r="L33" s="6" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="M33" s="6">
         <v>2427</v>
       </c>
       <c r="N33" s="6" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="O33" s="6">
         <v>0</v>
@@ -5157,13 +5155,13 @@
         <v>77</v>
       </c>
       <c r="R33" s="6" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="S33" s="6">
         <v>481</v>
       </c>
       <c r="T33" s="6" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="U33" s="6">
         <v>0</v>
@@ -5175,13 +5173,13 @@
         <v>70</v>
       </c>
       <c r="X33" s="6" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="Y33" s="6">
         <v>3631</v>
       </c>
       <c r="Z33" s="6" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="AA33" s="6">
         <v>0</v>
@@ -5195,16 +5193,16 @@
       <c r="AD33" s="6">
         <v>13343</v>
       </c>
-      <c r="AF33" s="9">
-        <v>46171</v>
-      </c>
-      <c r="AG33" s="5">
+      <c r="AH33" s="9">
+        <v>46154</v>
+      </c>
+      <c r="AI33" s="5">
         <v>1</v>
       </c>
     </row>
-    <row r="34" spans="1:33">
+    <row r="34" spans="1:35">
       <c r="A34" s="6" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="B34" s="6">
         <v>1639</v>
@@ -5213,37 +5211,37 @@
         <v>22379</v>
       </c>
       <c r="D34" s="6" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
       <c r="E34" s="6">
         <v>10953</v>
       </c>
       <c r="F34" s="6" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="G34" s="6">
         <v>415</v>
       </c>
       <c r="H34" s="6" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="I34" s="6">
         <v>1364</v>
       </c>
       <c r="J34" s="6" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="K34" s="6">
         <v>935</v>
       </c>
       <c r="L34" s="6" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="M34" s="6">
         <v>2356</v>
       </c>
       <c r="N34" s="6" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="O34" s="6">
         <v>0</v>
@@ -5255,13 +5253,13 @@
         <v>133</v>
       </c>
       <c r="R34" s="6" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="S34" s="6">
         <v>3138</v>
       </c>
       <c r="T34" s="6" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="U34" s="6">
         <v>0</v>
@@ -5273,13 +5271,13 @@
         <v>52</v>
       </c>
       <c r="X34" s="6" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
       <c r="Y34" s="6">
         <v>2560</v>
       </c>
       <c r="Z34" s="6" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="AA34" s="6">
         <v>0</v>
@@ -5293,16 +5291,16 @@
       <c r="AD34" s="6">
         <v>10953</v>
       </c>
-      <c r="AF34" s="9">
-        <v>46171</v>
-      </c>
-      <c r="AG34" s="5">
+      <c r="AH34" s="9">
+        <v>46154</v>
+      </c>
+      <c r="AI34" s="5">
         <v>1</v>
       </c>
     </row>
-    <row r="35" spans="1:33">
+    <row r="35" spans="1:35">
       <c r="A35" s="6" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="B35" s="6">
         <v>1629</v>
@@ -5311,19 +5309,19 @@
         <v>4994</v>
       </c>
       <c r="D35" s="6" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
       <c r="E35" s="6">
         <v>4994</v>
       </c>
       <c r="F35" s="6" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
       <c r="G35" s="6">
         <v>9</v>
       </c>
       <c r="H35" s="6" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="I35" s="6">
         <v>0</v>
@@ -5341,7 +5339,7 @@
         <v>2404</v>
       </c>
       <c r="N35" s="6" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
       <c r="O35" s="6">
         <v>0</v>
@@ -5377,7 +5375,7 @@
         <v>2581</v>
       </c>
       <c r="Z35" s="6" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="AA35" s="6">
         <v>0</v>
@@ -5391,16 +5389,16 @@
       <c r="AD35" s="6">
         <v>4994</v>
       </c>
-      <c r="AF35" s="9">
-        <v>46171</v>
-      </c>
-      <c r="AG35" s="5">
+      <c r="AH35" s="9">
+        <v>46154</v>
+      </c>
+      <c r="AI35" s="5">
         <v>1</v>
       </c>
     </row>
-    <row r="36" spans="1:33">
+    <row r="36" spans="1:35">
       <c r="A36" s="6" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="B36" s="6">
         <v>1616</v>
@@ -5409,19 +5407,19 @@
         <v>9</v>
       </c>
       <c r="D36" s="6" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="E36" s="6">
         <v>9</v>
       </c>
       <c r="F36" s="6" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="G36" s="6">
         <v>9</v>
       </c>
       <c r="H36" s="6" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="I36" s="6">
         <v>0</v>
@@ -5489,10 +5487,10 @@
       <c r="AD36" s="6">
         <v>9</v>
       </c>
-      <c r="AF36" s="9">
-        <v>46171</v>
-      </c>
-      <c r="AG36" s="5">
+      <c r="AH36" s="9">
+        <v>46154</v>
+      </c>
+      <c r="AI36" s="5">
         <v>1</v>
       </c>
     </row>
@@ -5513,21 +5511,21 @@
   <sheetData>
     <row r="1" spans="1:3">
       <c r="A1" t="s">
+        <v>307</v>
+      </c>
+      <c r="B1" t="s">
         <v>308</v>
       </c>
-      <c r="B1" t="s">
+      <c r="C1" t="s">
         <v>309</v>
-      </c>
-      <c r="C1" t="s">
-        <v>310</v>
       </c>
     </row>
     <row r="2" spans="1:3">
       <c r="A2" t="s">
-        <v>157</v>
+        <v>310</v>
       </c>
       <c r="B2" t="s">
-        <v>157</v>
+        <v>310</v>
       </c>
       <c r="C2">
         <v>1648</v>
@@ -5535,10 +5533,10 @@
     </row>
     <row r="3" spans="1:3">
       <c r="A3" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="B3" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="C3">
         <v>1636</v>
@@ -5546,10 +5544,10 @@
     </row>
     <row r="4" spans="1:3">
       <c r="A4" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="B4" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="C4">
         <v>1629</v>
@@ -5557,10 +5555,10 @@
     </row>
     <row r="5" spans="1:3">
       <c r="A5" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="B5" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="C5">
         <v>1639</v>
@@ -5568,10 +5566,10 @@
     </row>
     <row r="6" spans="1:3">
       <c r="A6" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="B6" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="C6">
         <v>1622</v>
@@ -5579,10 +5577,10 @@
     </row>
     <row r="7" spans="1:3">
       <c r="A7" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="B7" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="C7">
         <v>1652</v>
@@ -5590,10 +5588,10 @@
     </row>
     <row r="8" spans="1:3">
       <c r="A8" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="B8" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="C8">
         <v>1635</v>
@@ -5612,10 +5610,10 @@
     </row>
     <row r="10" spans="1:3">
       <c r="A10" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="B10" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="C10">
         <v>1624</v>
@@ -5634,10 +5632,10 @@
     </row>
     <row r="12" spans="1:3">
       <c r="A12" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="B12" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="C12">
         <v>1628</v>
@@ -5678,10 +5676,10 @@
     </row>
     <row r="16" spans="1:3">
       <c r="A16" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="B16" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="C16">
         <v>1642</v>
@@ -5689,10 +5687,10 @@
     </row>
     <row r="17" spans="1:3">
       <c r="A17" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="B17" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="C17">
         <v>1647</v>
@@ -5722,10 +5720,10 @@
     </row>
     <row r="20" spans="1:3">
       <c r="A20" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="B20" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="C20">
         <v>1651</v>
@@ -5744,10 +5742,10 @@
     </row>
     <row r="22" spans="1:3">
       <c r="A22" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="B22" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="C22">
         <v>1632</v>
@@ -5755,10 +5753,10 @@
     </row>
     <row r="23" spans="1:3">
       <c r="A23" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="B23" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="C23">
         <v>1616</v>
@@ -5777,10 +5775,10 @@
     </row>
     <row r="25" spans="1:3">
       <c r="A25" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="B25" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="C25">
         <v>1630</v>
@@ -5799,10 +5797,10 @@
     </row>
     <row r="27" spans="1:3">
       <c r="A27" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="B27" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="C27">
         <v>1653</v>
@@ -5843,10 +5841,10 @@
     </row>
     <row r="31" spans="1:3">
       <c r="A31" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="B31" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="C31">
         <v>1641</v>
@@ -5887,10 +5885,10 @@
     </row>
     <row r="35" spans="1:3">
       <c r="A35" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
       <c r="B35" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
       <c r="C35">
         <v>1621</v>
@@ -5974,38 +5972,38 @@
       </c>
     </row>
     <row r="2" spans="1:18">
-      <c r="A2" s="3" t="str">
-        <f>DAY(VLOOKUP(C2,Pasted!$A$3:$AF$50,32,0))&amp;" "&amp;CHOOSE(MONTH(VLOOKUP(C2,Pasted!$A$3:$AF$50,32,0)),"Jan","Feb","Mar","Apr","May","Jun","Jul","Aug","Sep","Oct","Nov","Dec")&amp;" "&amp;YEAR(VLOOKUP(C2,Pasted!$A$3:$AF$50,32,0))</f>
-        <v>29 May 2026</v>
+      <c r="A2" s="3" t="e">
+        <f>DAY(VLOOKUP(C2,Pasted!$A$3:$AH$50,34,0))&amp;" "&amp;CHOOSE(MONTH(VLOOKUP(C2,Pasted!$A$3:$AH$50,34,0)),"Jan","Feb","Mar","Apr","May","Jun","Jul","Aug","Sep","Oct","Nov","Dec")&amp;" "&amp;YEAR(VLOOKUP(C2,Pasted!$A$3:$AH$50,34,0))</f>
+        <v>#N/A</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>157</v>
+        <v>310</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>157</v>
+        <v>310</v>
       </c>
       <c r="D2" s="1">
         <v>1648</v>
       </c>
       <c r="E2" s="1">
         <f>IFERROR(VLOOKUP(C2,Pasted!$A$3:$AD$50,3,0),0)</f>
-        <v>34479</v>
+        <v>0</v>
       </c>
       <c r="F2" s="1">
         <f>IFERROR(VLOOKUP(C2,Pasted!$A$3:$AD$50,7,0),0)</f>
-        <v>3754</v>
+        <v>0</v>
       </c>
       <c r="G2" s="1">
         <f>IFERROR(VLOOKUP(C2,Pasted!$A$3:$AD$50,9,0),0)</f>
-        <v>1598</v>
+        <v>0</v>
       </c>
       <c r="H2" s="1">
         <f>IFERROR(VLOOKUP(C2,Pasted!$A$3:$AD$50,11,0),0)</f>
-        <v>2869</v>
+        <v>0</v>
       </c>
       <c r="I2" s="1">
         <f>IFERROR(VLOOKUP(C2,Pasted!$A$3:$AD$50,13,0),0)</f>
-        <v>2409</v>
+        <v>0</v>
       </c>
       <c r="J2" s="1">
         <f>IFERROR(VLOOKUP(C2,Pasted!$A$3:$AD$50,15,0),0)</f>
@@ -6013,11 +6011,11 @@
       </c>
       <c r="K2" s="1">
         <f>IFERROR(VLOOKUP(C2,Pasted!$A$3:$AD$50,17,0),0)</f>
-        <v>594</v>
+        <v>0</v>
       </c>
       <c r="L2" s="1">
         <f>IFERROR(VLOOKUP(C2,Pasted!$A$3:$AD$50,19,0),0)</f>
-        <v>10087</v>
+        <v>0</v>
       </c>
       <c r="M2" s="1">
         <f>IFERROR(VLOOKUP(C2,Pasted!$A$3:$AD$50,21,0),0)</f>
@@ -6038,21 +6036,21 @@
       <c r="Q2" s="1" t="s">
         <v>329</v>
       </c>
-      <c r="R2" s="1">
-        <f>IF(OR(VLOOKUP(C2,Pasted!$A$3:$AG$50,33,0)=1,LOWER(VLOOKUP(C2,Pasted!$A$3:$AG$50,33,0))="weekday"),1,0)</f>
-        <v>1</v>
+      <c r="R2" s="1" t="e">
+        <f>IF(OR(VLOOKUP(C2,Pasted!$A$3:$AI$50,35,0)=1,LOWER(VLOOKUP(C2,Pasted!$A$3:$AI$50,35,0))="weekday",LOWER(VLOOKUP(C2,Pasted!$A$3:$AI$50,35,0))="yes"),1,0)</f>
+        <v>#N/A</v>
       </c>
     </row>
     <row r="3" spans="1:18">
       <c r="A3" s="3" t="str">
-        <f>DAY(VLOOKUP(C3,Pasted!$A$3:$AF$50,32,0))&amp;" "&amp;CHOOSE(MONTH(VLOOKUP(C3,Pasted!$A$3:$AF$50,32,0)),"Jan","Feb","Mar","Apr","May","Jun","Jul","Aug","Sep","Oct","Nov","Dec")&amp;" "&amp;YEAR(VLOOKUP(C3,Pasted!$A$3:$AF$50,32,0))</f>
-        <v>29 May 2026</v>
+        <f>DAY(VLOOKUP(C3,Pasted!$A$3:$AH$50,34,0))&amp;" "&amp;CHOOSE(MONTH(VLOOKUP(C3,Pasted!$A$3:$AH$50,34,0)),"Jan","Feb","Mar","Apr","May","Jun","Jul","Aug","Sep","Oct","Nov","Dec")&amp;" "&amp;YEAR(VLOOKUP(C3,Pasted!$A$3:$AH$50,34,0))</f>
+        <v>12 May 2026</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="D3" s="1">
         <v>1636</v>
@@ -6062,8 +6060,8 @@
         <v>35902</v>
       </c>
       <c r="F3" s="1">
-        <f>IFERROR(VLOOKUP(C3,Pasted!$A$3:$AD$50,5,0),0)</f>
-        <v>18984</v>
+        <f>IFERROR(VLOOKUP(C3,Pasted!$A$3:$AD$50,7,0),0)</f>
+        <v>3044</v>
       </c>
       <c r="G3" s="1">
         <f>IFERROR(VLOOKUP(C3,Pasted!$A$3:$AD$50,9,0),0)</f>
@@ -6109,20 +6107,20 @@
         <v>329</v>
       </c>
       <c r="R3" s="1">
-        <f>IF(OR(VLOOKUP(C3,Pasted!$A$3:$AG$50,33,0)=1,LOWER(VLOOKUP(C3,Pasted!$A$3:$AG$50,33,0))="weekday"),1,0)</f>
+        <f>IF(OR(VLOOKUP(C3,Pasted!$A$3:$AI$50,35,0)=1,LOWER(VLOOKUP(C3,Pasted!$A$3:$AI$50,35,0))="weekday",LOWER(VLOOKUP(C3,Pasted!$A$3:$AI$50,35,0))="yes"),1,0)</f>
         <v>1</v>
       </c>
     </row>
     <row r="4" spans="1:18">
       <c r="A4" s="3" t="str">
-        <f>DAY(VLOOKUP(C4,Pasted!$A$3:$AF$50,32,0))&amp;" "&amp;CHOOSE(MONTH(VLOOKUP(C4,Pasted!$A$3:$AF$50,32,0)),"Jan","Feb","Mar","Apr","May","Jun","Jul","Aug","Sep","Oct","Nov","Dec")&amp;" "&amp;YEAR(VLOOKUP(C4,Pasted!$A$3:$AF$50,32,0))</f>
-        <v>29 May 2026</v>
+        <f>DAY(VLOOKUP(C4,Pasted!$A$3:$AH$50,34,0))&amp;" "&amp;CHOOSE(MONTH(VLOOKUP(C4,Pasted!$A$3:$AH$50,34,0)),"Jan","Feb","Mar","Apr","May","Jun","Jul","Aug","Sep","Oct","Nov","Dec")&amp;" "&amp;YEAR(VLOOKUP(C4,Pasted!$A$3:$AH$50,34,0))</f>
+        <v>12 May 2026</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="D4" s="1">
         <v>1629</v>
@@ -6132,8 +6130,8 @@
         <v>4994</v>
       </c>
       <c r="F4" s="1">
-        <f>IFERROR(VLOOKUP(C4,Pasted!$A$3:$AD$50,5,0),0)</f>
-        <v>4994</v>
+        <f>IFERROR(VLOOKUP(C4,Pasted!$A$3:$AD$50,7,0),0)</f>
+        <v>9</v>
       </c>
       <c r="G4" s="1">
         <f>IFERROR(VLOOKUP(C4,Pasted!$A$3:$AD$50,9,0),0)</f>
@@ -6179,20 +6177,20 @@
         <v>329</v>
       </c>
       <c r="R4" s="1">
-        <f>IF(OR(VLOOKUP(C4,Pasted!$A$3:$AG$50,33,0)=1,LOWER(VLOOKUP(C4,Pasted!$A$3:$AG$50,33,0))="weekday"),1,0)</f>
+        <f>IF(OR(VLOOKUP(C4,Pasted!$A$3:$AI$50,35,0)=1,LOWER(VLOOKUP(C4,Pasted!$A$3:$AI$50,35,0))="weekday",LOWER(VLOOKUP(C4,Pasted!$A$3:$AI$50,35,0))="yes"),1,0)</f>
         <v>1</v>
       </c>
     </row>
     <row r="5" spans="1:18">
       <c r="A5" s="3" t="str">
-        <f>DAY(VLOOKUP(C5,Pasted!$A$3:$AF$50,32,0))&amp;" "&amp;CHOOSE(MONTH(VLOOKUP(C5,Pasted!$A$3:$AF$50,32,0)),"Jan","Feb","Mar","Apr","May","Jun","Jul","Aug","Sep","Oct","Nov","Dec")&amp;" "&amp;YEAR(VLOOKUP(C5,Pasted!$A$3:$AF$50,32,0))</f>
-        <v>29 May 2026</v>
+        <f>DAY(VLOOKUP(C5,Pasted!$A$3:$AH$50,34,0))&amp;" "&amp;CHOOSE(MONTH(VLOOKUP(C5,Pasted!$A$3:$AH$50,34,0)),"Jan","Feb","Mar","Apr","May","Jun","Jul","Aug","Sep","Oct","Nov","Dec")&amp;" "&amp;YEAR(VLOOKUP(C5,Pasted!$A$3:$AH$50,34,0))</f>
+        <v>12 May 2026</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="D5" s="1">
         <v>1639</v>
@@ -6202,8 +6200,8 @@
         <v>22379</v>
       </c>
       <c r="F5" s="1">
-        <f>IFERROR(VLOOKUP(C5,Pasted!$A$3:$AD$50,5,0),0)</f>
-        <v>10953</v>
+        <f>IFERROR(VLOOKUP(C5,Pasted!$A$3:$AD$50,7,0),0)</f>
+        <v>415</v>
       </c>
       <c r="G5" s="1">
         <f>IFERROR(VLOOKUP(C5,Pasted!$A$3:$AD$50,9,0),0)</f>
@@ -6249,20 +6247,20 @@
         <v>329</v>
       </c>
       <c r="R5" s="1">
-        <f>IF(OR(VLOOKUP(C5,Pasted!$A$3:$AG$50,33,0)=1,LOWER(VLOOKUP(C5,Pasted!$A$3:$AG$50,33,0))="weekday"),1,0)</f>
+        <f>IF(OR(VLOOKUP(C5,Pasted!$A$3:$AI$50,35,0)=1,LOWER(VLOOKUP(C5,Pasted!$A$3:$AI$50,35,0))="weekday",LOWER(VLOOKUP(C5,Pasted!$A$3:$AI$50,35,0))="yes"),1,0)</f>
         <v>1</v>
       </c>
     </row>
     <row r="6" spans="1:18">
       <c r="A6" s="3" t="str">
-        <f>DAY(VLOOKUP(C6,Pasted!$A$3:$AF$50,32,0))&amp;" "&amp;CHOOSE(MONTH(VLOOKUP(C6,Pasted!$A$3:$AF$50,32,0)),"Jan","Feb","Mar","Apr","May","Jun","Jul","Aug","Sep","Oct","Nov","Dec")&amp;" "&amp;YEAR(VLOOKUP(C6,Pasted!$A$3:$AF$50,32,0))</f>
-        <v>29 May 2026</v>
+        <f>DAY(VLOOKUP(C6,Pasted!$A$3:$AH$50,34,0))&amp;" "&amp;CHOOSE(MONTH(VLOOKUP(C6,Pasted!$A$3:$AH$50,34,0)),"Jan","Feb","Mar","Apr","May","Jun","Jul","Aug","Sep","Oct","Nov","Dec")&amp;" "&amp;YEAR(VLOOKUP(C6,Pasted!$A$3:$AH$50,34,0))</f>
+        <v>12 May 2026</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="D6" s="1">
         <v>1622</v>
@@ -6272,8 +6270,8 @@
         <v>32399</v>
       </c>
       <c r="F6" s="1">
-        <f>IFERROR(VLOOKUP(C6,Pasted!$A$3:$AD$50,5,0),0)</f>
-        <v>17316</v>
+        <f>IFERROR(VLOOKUP(C6,Pasted!$A$3:$AD$50,7,0),0)</f>
+        <v>2015</v>
       </c>
       <c r="G6" s="1">
         <f>IFERROR(VLOOKUP(C6,Pasted!$A$3:$AD$50,9,0),0)</f>
@@ -6319,20 +6317,20 @@
         <v>329</v>
       </c>
       <c r="R6" s="1">
-        <f>IF(OR(VLOOKUP(C6,Pasted!$A$3:$AG$50,33,0)=1,LOWER(VLOOKUP(C6,Pasted!$A$3:$AG$50,33,0))="weekday"),1,0)</f>
+        <f>IF(OR(VLOOKUP(C6,Pasted!$A$3:$AI$50,35,0)=1,LOWER(VLOOKUP(C6,Pasted!$A$3:$AI$50,35,0))="weekday",LOWER(VLOOKUP(C6,Pasted!$A$3:$AI$50,35,0))="yes"),1,0)</f>
         <v>1</v>
       </c>
     </row>
     <row r="7" spans="1:18">
       <c r="A7" s="3" t="str">
-        <f>DAY(VLOOKUP(C7,Pasted!$A$3:$AF$50,32,0))&amp;" "&amp;CHOOSE(MONTH(VLOOKUP(C7,Pasted!$A$3:$AF$50,32,0)),"Jan","Feb","Mar","Apr","May","Jun","Jul","Aug","Sep","Oct","Nov","Dec")&amp;" "&amp;YEAR(VLOOKUP(C7,Pasted!$A$3:$AF$50,32,0))</f>
-        <v>29 May 2026</v>
+        <f>DAY(VLOOKUP(C7,Pasted!$A$3:$AH$50,34,0))&amp;" "&amp;CHOOSE(MONTH(VLOOKUP(C7,Pasted!$A$3:$AH$50,34,0)),"Jan","Feb","Mar","Apr","May","Jun","Jul","Aug","Sep","Oct","Nov","Dec")&amp;" "&amp;YEAR(VLOOKUP(C7,Pasted!$A$3:$AH$50,34,0))</f>
+        <v>12 May 2026</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="D7" s="1">
         <v>1652</v>
@@ -6342,8 +6340,8 @@
         <v>23102</v>
       </c>
       <c r="F7" s="1">
-        <f>IFERROR(VLOOKUP(C7,Pasted!$A$3:$AD$50,5,0),0)</f>
-        <v>13628</v>
+        <f>IFERROR(VLOOKUP(C7,Pasted!$A$3:$AD$50,7,0),0)</f>
+        <v>620</v>
       </c>
       <c r="G7" s="1">
         <f>IFERROR(VLOOKUP(C7,Pasted!$A$3:$AD$50,9,0),0)</f>
@@ -6389,20 +6387,20 @@
         <v>329</v>
       </c>
       <c r="R7" s="1">
-        <f>IF(OR(VLOOKUP(C7,Pasted!$A$3:$AG$50,33,0)=1,LOWER(VLOOKUP(C7,Pasted!$A$3:$AG$50,33,0))="weekday"),1,0)</f>
+        <f>IF(OR(VLOOKUP(C7,Pasted!$A$3:$AI$50,35,0)=1,LOWER(VLOOKUP(C7,Pasted!$A$3:$AI$50,35,0))="weekday",LOWER(VLOOKUP(C7,Pasted!$A$3:$AI$50,35,0))="yes"),1,0)</f>
         <v>1</v>
       </c>
     </row>
     <row r="8" spans="1:18">
       <c r="A8" s="3" t="str">
-        <f>DAY(VLOOKUP(C8,Pasted!$A$3:$AF$50,32,0))&amp;" "&amp;CHOOSE(MONTH(VLOOKUP(C8,Pasted!$A$3:$AF$50,32,0)),"Jan","Feb","Mar","Apr","May","Jun","Jul","Aug","Sep","Oct","Nov","Dec")&amp;" "&amp;YEAR(VLOOKUP(C8,Pasted!$A$3:$AF$50,32,0))</f>
-        <v>29 May 2026</v>
+        <f>DAY(VLOOKUP(C8,Pasted!$A$3:$AH$50,34,0))&amp;" "&amp;CHOOSE(MONTH(VLOOKUP(C8,Pasted!$A$3:$AH$50,34,0)),"Jan","Feb","Mar","Apr","May","Jun","Jul","Aug","Sep","Oct","Nov","Dec")&amp;" "&amp;YEAR(VLOOKUP(C8,Pasted!$A$3:$AH$50,34,0))</f>
+        <v>12 May 2026</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="D8" s="1">
         <v>1635</v>
@@ -6412,8 +6410,8 @@
         <v>33658</v>
       </c>
       <c r="F8" s="1">
-        <f>IFERROR(VLOOKUP(C8,Pasted!$A$3:$AD$50,5,0),0)</f>
-        <v>19227</v>
+        <f>IFERROR(VLOOKUP(C8,Pasted!$A$3:$AD$50,7,0),0)</f>
+        <v>1291</v>
       </c>
       <c r="G8" s="1">
         <f>IFERROR(VLOOKUP(C8,Pasted!$A$3:$AD$50,9,0),0)</f>
@@ -6459,14 +6457,14 @@
         <v>329</v>
       </c>
       <c r="R8" s="1">
-        <f>IF(OR(VLOOKUP(C8,Pasted!$A$3:$AG$50,33,0)=1,LOWER(VLOOKUP(C8,Pasted!$A$3:$AG$50,33,0))="weekday"),1,0)</f>
+        <f>IF(OR(VLOOKUP(C8,Pasted!$A$3:$AI$50,35,0)=1,LOWER(VLOOKUP(C8,Pasted!$A$3:$AI$50,35,0))="weekday",LOWER(VLOOKUP(C8,Pasted!$A$3:$AI$50,35,0))="yes"),1,0)</f>
         <v>1</v>
       </c>
     </row>
     <row r="9" spans="1:18">
       <c r="A9" s="3" t="str">
-        <f>DAY(VLOOKUP(C9,Pasted!$A$3:$AF$50,32,0))&amp;" "&amp;CHOOSE(MONTH(VLOOKUP(C9,Pasted!$A$3:$AF$50,32,0)),"Jan","Feb","Mar","Apr","May","Jun","Jul","Aug","Sep","Oct","Nov","Dec")&amp;" "&amp;YEAR(VLOOKUP(C9,Pasted!$A$3:$AF$50,32,0))</f>
-        <v>29 May 2026</v>
+        <f>DAY(VLOOKUP(C9,Pasted!$A$3:$AH$50,34,0))&amp;" "&amp;CHOOSE(MONTH(VLOOKUP(C9,Pasted!$A$3:$AH$50,34,0)),"Jan","Feb","Mar","Apr","May","Jun","Jul","Aug","Sep","Oct","Nov","Dec")&amp;" "&amp;YEAR(VLOOKUP(C9,Pasted!$A$3:$AH$50,34,0))</f>
+        <v>12 May 2026</v>
       </c>
       <c r="B9" s="1" t="s">
         <v>40</v>
@@ -6482,8 +6480,8 @@
         <v>34060</v>
       </c>
       <c r="F9" s="1">
-        <f>IFERROR(VLOOKUP(C9,Pasted!$A$3:$AD$50,5,0),0)</f>
-        <v>34060</v>
+        <f>IFERROR(VLOOKUP(C9,Pasted!$A$3:$AD$50,7,0),0)</f>
+        <v>5</v>
       </c>
       <c r="G9" s="1">
         <f>IFERROR(VLOOKUP(C9,Pasted!$A$3:$AD$50,9,0),0)</f>
@@ -6529,20 +6527,20 @@
         <v>329</v>
       </c>
       <c r="R9" s="1">
-        <f>IF(OR(VLOOKUP(C9,Pasted!$A$3:$AG$50,33,0)=1,LOWER(VLOOKUP(C9,Pasted!$A$3:$AG$50,33,0))="weekday"),1,0)</f>
+        <f>IF(OR(VLOOKUP(C9,Pasted!$A$3:$AI$50,35,0)=1,LOWER(VLOOKUP(C9,Pasted!$A$3:$AI$50,35,0))="weekday",LOWER(VLOOKUP(C9,Pasted!$A$3:$AI$50,35,0))="yes"),1,0)</f>
         <v>1</v>
       </c>
     </row>
     <row r="10" spans="1:18">
       <c r="A10" s="3" t="str">
-        <f>DAY(VLOOKUP(C10,Pasted!$A$3:$AF$50,32,0))&amp;" "&amp;CHOOSE(MONTH(VLOOKUP(C10,Pasted!$A$3:$AF$50,32,0)),"Jan","Feb","Mar","Apr","May","Jun","Jul","Aug","Sep","Oct","Nov","Dec")&amp;" "&amp;YEAR(VLOOKUP(C10,Pasted!$A$3:$AF$50,32,0))</f>
-        <v>29 May 2026</v>
+        <f>DAY(VLOOKUP(C10,Pasted!$A$3:$AH$50,34,0))&amp;" "&amp;CHOOSE(MONTH(VLOOKUP(C10,Pasted!$A$3:$AH$50,34,0)),"Jan","Feb","Mar","Apr","May","Jun","Jul","Aug","Sep","Oct","Nov","Dec")&amp;" "&amp;YEAR(VLOOKUP(C10,Pasted!$A$3:$AH$50,34,0))</f>
+        <v>12 May 2026</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="D10" s="1">
         <v>1624</v>
@@ -6552,8 +6550,8 @@
         <v>35162</v>
       </c>
       <c r="F10" s="1">
-        <f>IFERROR(VLOOKUP(C10,Pasted!$A$3:$AD$50,5,0),0)</f>
-        <v>17640</v>
+        <f>IFERROR(VLOOKUP(C10,Pasted!$A$3:$AD$50,7,0),0)</f>
+        <v>2152</v>
       </c>
       <c r="G10" s="1">
         <f>IFERROR(VLOOKUP(C10,Pasted!$A$3:$AD$50,9,0),0)</f>
@@ -6599,14 +6597,14 @@
         <v>329</v>
       </c>
       <c r="R10" s="1">
-        <f>IF(OR(VLOOKUP(C10,Pasted!$A$3:$AG$50,33,0)=1,LOWER(VLOOKUP(C10,Pasted!$A$3:$AG$50,33,0))="weekday"),1,0)</f>
+        <f>IF(OR(VLOOKUP(C10,Pasted!$A$3:$AI$50,35,0)=1,LOWER(VLOOKUP(C10,Pasted!$A$3:$AI$50,35,0))="weekday",LOWER(VLOOKUP(C10,Pasted!$A$3:$AI$50,35,0))="yes"),1,0)</f>
         <v>1</v>
       </c>
     </row>
     <row r="11" spans="1:18">
       <c r="A11" s="3" t="str">
-        <f>DAY(VLOOKUP(C11,Pasted!$A$3:$AF$50,32,0))&amp;" "&amp;CHOOSE(MONTH(VLOOKUP(C11,Pasted!$A$3:$AF$50,32,0)),"Jan","Feb","Mar","Apr","May","Jun","Jul","Aug","Sep","Oct","Nov","Dec")&amp;" "&amp;YEAR(VLOOKUP(C11,Pasted!$A$3:$AF$50,32,0))</f>
-        <v>29 May 2026</v>
+        <f>DAY(VLOOKUP(C11,Pasted!$A$3:$AH$50,34,0))&amp;" "&amp;CHOOSE(MONTH(VLOOKUP(C11,Pasted!$A$3:$AH$50,34,0)),"Jan","Feb","Mar","Apr","May","Jun","Jul","Aug","Sep","Oct","Nov","Dec")&amp;" "&amp;YEAR(VLOOKUP(C11,Pasted!$A$3:$AH$50,34,0))</f>
+        <v>12 May 2026</v>
       </c>
       <c r="B11" s="1" t="s">
         <v>64</v>
@@ -6622,8 +6620,8 @@
         <v>33057</v>
       </c>
       <c r="F11" s="1">
-        <f>IFERROR(VLOOKUP(C11,Pasted!$A$3:$AD$50,5,0),0)</f>
-        <v>33057</v>
+        <f>IFERROR(VLOOKUP(C11,Pasted!$A$3:$AD$50,7,0),0)</f>
+        <v>5</v>
       </c>
       <c r="G11" s="1">
         <f>IFERROR(VLOOKUP(C11,Pasted!$A$3:$AD$50,9,0),0)</f>
@@ -6669,20 +6667,20 @@
         <v>329</v>
       </c>
       <c r="R11" s="1">
-        <f>IF(OR(VLOOKUP(C11,Pasted!$A$3:$AG$50,33,0)=1,LOWER(VLOOKUP(C11,Pasted!$A$3:$AG$50,33,0))="weekday"),1,0)</f>
+        <f>IF(OR(VLOOKUP(C11,Pasted!$A$3:$AI$50,35,0)=1,LOWER(VLOOKUP(C11,Pasted!$A$3:$AI$50,35,0))="weekday",LOWER(VLOOKUP(C11,Pasted!$A$3:$AI$50,35,0))="yes"),1,0)</f>
         <v>1</v>
       </c>
     </row>
     <row r="12" spans="1:18">
       <c r="A12" s="3" t="str">
-        <f>DAY(VLOOKUP(C12,Pasted!$A$3:$AF$50,32,0))&amp;" "&amp;CHOOSE(MONTH(VLOOKUP(C12,Pasted!$A$3:$AF$50,32,0)),"Jan","Feb","Mar","Apr","May","Jun","Jul","Aug","Sep","Oct","Nov","Dec")&amp;" "&amp;YEAR(VLOOKUP(C12,Pasted!$A$3:$AF$50,32,0))</f>
-        <v>29 May 2026</v>
+        <f>DAY(VLOOKUP(C12,Pasted!$A$3:$AH$50,34,0))&amp;" "&amp;CHOOSE(MONTH(VLOOKUP(C12,Pasted!$A$3:$AH$50,34,0)),"Jan","Feb","Mar","Apr","May","Jun","Jul","Aug","Sep","Oct","Nov","Dec")&amp;" "&amp;YEAR(VLOOKUP(C12,Pasted!$A$3:$AH$50,34,0))</f>
+        <v>12 May 2026</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="D12" s="1">
         <v>1628</v>
@@ -6692,8 +6690,8 @@
         <v>33332</v>
       </c>
       <c r="F12" s="1">
-        <f>IFERROR(VLOOKUP(C12,Pasted!$A$3:$AD$50,5,0),0)</f>
-        <v>19461</v>
+        <f>IFERROR(VLOOKUP(C12,Pasted!$A$3:$AD$50,7,0),0)</f>
+        <v>943</v>
       </c>
       <c r="G12" s="1">
         <f>IFERROR(VLOOKUP(C12,Pasted!$A$3:$AD$50,9,0),0)</f>
@@ -6739,14 +6737,14 @@
         <v>329</v>
       </c>
       <c r="R12" s="1">
-        <f>IF(OR(VLOOKUP(C12,Pasted!$A$3:$AG$50,33,0)=1,LOWER(VLOOKUP(C12,Pasted!$A$3:$AG$50,33,0))="weekday"),1,0)</f>
+        <f>IF(OR(VLOOKUP(C12,Pasted!$A$3:$AI$50,35,0)=1,LOWER(VLOOKUP(C12,Pasted!$A$3:$AI$50,35,0))="weekday",LOWER(VLOOKUP(C12,Pasted!$A$3:$AI$50,35,0))="yes"),1,0)</f>
         <v>1</v>
       </c>
     </row>
     <row r="13" spans="1:18">
       <c r="A13" s="3" t="str">
-        <f>DAY(VLOOKUP(C13,Pasted!$A$3:$AF$50,32,0))&amp;" "&amp;CHOOSE(MONTH(VLOOKUP(C13,Pasted!$A$3:$AF$50,32,0)),"Jan","Feb","Mar","Apr","May","Jun","Jul","Aug","Sep","Oct","Nov","Dec")&amp;" "&amp;YEAR(VLOOKUP(C13,Pasted!$A$3:$AF$50,32,0))</f>
-        <v>29 May 2026</v>
+        <f>DAY(VLOOKUP(C13,Pasted!$A$3:$AH$50,34,0))&amp;" "&amp;CHOOSE(MONTH(VLOOKUP(C13,Pasted!$A$3:$AH$50,34,0)),"Jan","Feb","Mar","Apr","May","Jun","Jul","Aug","Sep","Oct","Nov","Dec")&amp;" "&amp;YEAR(VLOOKUP(C13,Pasted!$A$3:$AH$50,34,0))</f>
+        <v>12 May 2026</v>
       </c>
       <c r="B13" s="1" t="s">
         <v>81</v>
@@ -6762,8 +6760,8 @@
         <v>39426</v>
       </c>
       <c r="F13" s="1">
-        <f>IFERROR(VLOOKUP(C13,Pasted!$A$3:$AD$50,5,0),0)</f>
-        <v>28830</v>
+        <f>IFERROR(VLOOKUP(C13,Pasted!$A$3:$AD$50,7,0),0)</f>
+        <v>1233</v>
       </c>
       <c r="G13" s="1">
         <f>IFERROR(VLOOKUP(C13,Pasted!$A$3:$AD$50,9,0),0)</f>
@@ -6809,14 +6807,14 @@
         <v>329</v>
       </c>
       <c r="R13" s="1">
-        <f>IF(OR(VLOOKUP(C13,Pasted!$A$3:$AG$50,33,0)=1,LOWER(VLOOKUP(C13,Pasted!$A$3:$AG$50,33,0))="weekday"),1,0)</f>
+        <f>IF(OR(VLOOKUP(C13,Pasted!$A$3:$AI$50,35,0)=1,LOWER(VLOOKUP(C13,Pasted!$A$3:$AI$50,35,0))="weekday",LOWER(VLOOKUP(C13,Pasted!$A$3:$AI$50,35,0))="yes"),1,0)</f>
         <v>1</v>
       </c>
     </row>
     <row r="14" spans="1:18">
       <c r="A14" s="3" t="str">
-        <f>DAY(VLOOKUP(C14,Pasted!$A$3:$AF$50,32,0))&amp;" "&amp;CHOOSE(MONTH(VLOOKUP(C14,Pasted!$A$3:$AF$50,32,0)),"Jan","Feb","Mar","Apr","May","Jun","Jul","Aug","Sep","Oct","Nov","Dec")&amp;" "&amp;YEAR(VLOOKUP(C14,Pasted!$A$3:$AF$50,32,0))</f>
-        <v>29 May 2026</v>
+        <f>DAY(VLOOKUP(C14,Pasted!$A$3:$AH$50,34,0))&amp;" "&amp;CHOOSE(MONTH(VLOOKUP(C14,Pasted!$A$3:$AH$50,34,0)),"Jan","Feb","Mar","Apr","May","Jun","Jul","Aug","Sep","Oct","Nov","Dec")&amp;" "&amp;YEAR(VLOOKUP(C14,Pasted!$A$3:$AH$50,34,0))</f>
+        <v>12 May 2026</v>
       </c>
       <c r="B14" s="1" t="s">
         <v>102</v>
@@ -6832,8 +6830,8 @@
         <v>35641</v>
       </c>
       <c r="F14" s="1">
-        <f>IFERROR(VLOOKUP(C14,Pasted!$A$3:$AD$50,5,0),0)</f>
-        <v>27007</v>
+        <f>IFERROR(VLOOKUP(C14,Pasted!$A$3:$AD$50,7,0),0)</f>
+        <v>2313</v>
       </c>
       <c r="G14" s="1">
         <f>IFERROR(VLOOKUP(C14,Pasted!$A$3:$AD$50,9,0),0)</f>
@@ -6879,14 +6877,14 @@
         <v>329</v>
       </c>
       <c r="R14" s="1">
-        <f>IF(OR(VLOOKUP(C14,Pasted!$A$3:$AG$50,33,0)=1,LOWER(VLOOKUP(C14,Pasted!$A$3:$AG$50,33,0))="weekday"),1,0)</f>
+        <f>IF(OR(VLOOKUP(C14,Pasted!$A$3:$AI$50,35,0)=1,LOWER(VLOOKUP(C14,Pasted!$A$3:$AI$50,35,0))="weekday",LOWER(VLOOKUP(C14,Pasted!$A$3:$AI$50,35,0))="yes"),1,0)</f>
         <v>1</v>
       </c>
     </row>
     <row r="15" spans="1:18">
       <c r="A15" s="3" t="str">
-        <f>DAY(VLOOKUP(C15,Pasted!$A$3:$AF$50,32,0))&amp;" "&amp;CHOOSE(MONTH(VLOOKUP(C15,Pasted!$A$3:$AF$50,32,0)),"Jan","Feb","Mar","Apr","May","Jun","Jul","Aug","Sep","Oct","Nov","Dec")&amp;" "&amp;YEAR(VLOOKUP(C15,Pasted!$A$3:$AF$50,32,0))</f>
-        <v>29 May 2026</v>
+        <f>DAY(VLOOKUP(C15,Pasted!$A$3:$AH$50,34,0))&amp;" "&amp;CHOOSE(MONTH(VLOOKUP(C15,Pasted!$A$3:$AH$50,34,0)),"Jan","Feb","Mar","Apr","May","Jun","Jul","Aug","Sep","Oct","Nov","Dec")&amp;" "&amp;YEAR(VLOOKUP(C15,Pasted!$A$3:$AH$50,34,0))</f>
+        <v>12 May 2026</v>
       </c>
       <c r="B15" s="1" t="s">
         <v>139</v>
@@ -6902,8 +6900,8 @@
         <v>34458</v>
       </c>
       <c r="F15" s="1">
-        <f>IFERROR(VLOOKUP(C15,Pasted!$A$3:$AD$50,5,0),0)</f>
-        <v>21879</v>
+        <f>IFERROR(VLOOKUP(C15,Pasted!$A$3:$AD$50,7,0),0)</f>
+        <v>4623</v>
       </c>
       <c r="G15" s="1">
         <f>IFERROR(VLOOKUP(C15,Pasted!$A$3:$AD$50,9,0),0)</f>
@@ -6949,20 +6947,20 @@
         <v>329</v>
       </c>
       <c r="R15" s="1">
-        <f>IF(OR(VLOOKUP(C15,Pasted!$A$3:$AG$50,33,0)=1,LOWER(VLOOKUP(C15,Pasted!$A$3:$AG$50,33,0))="weekday"),1,0)</f>
+        <f>IF(OR(VLOOKUP(C15,Pasted!$A$3:$AI$50,35,0)=1,LOWER(VLOOKUP(C15,Pasted!$A$3:$AI$50,35,0))="weekday",LOWER(VLOOKUP(C15,Pasted!$A$3:$AI$50,35,0))="yes"),1,0)</f>
         <v>1</v>
       </c>
     </row>
     <row r="16" spans="1:18">
       <c r="A16" s="3" t="str">
-        <f>DAY(VLOOKUP(C16,Pasted!$A$3:$AF$50,32,0))&amp;" "&amp;CHOOSE(MONTH(VLOOKUP(C16,Pasted!$A$3:$AF$50,32,0)),"Jan","Feb","Mar","Apr","May","Jun","Jul","Aug","Sep","Oct","Nov","Dec")&amp;" "&amp;YEAR(VLOOKUP(C16,Pasted!$A$3:$AF$50,32,0))</f>
-        <v>29 May 2026</v>
+        <f>DAY(VLOOKUP(C16,Pasted!$A$3:$AH$50,34,0))&amp;" "&amp;CHOOSE(MONTH(VLOOKUP(C16,Pasted!$A$3:$AH$50,34,0)),"Jan","Feb","Mar","Apr","May","Jun","Jul","Aug","Sep","Oct","Nov","Dec")&amp;" "&amp;YEAR(VLOOKUP(C16,Pasted!$A$3:$AH$50,34,0))</f>
+        <v>12 May 2026</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="D16" s="1">
         <v>1642</v>
@@ -6972,8 +6970,8 @@
         <v>34106</v>
       </c>
       <c r="F16" s="1">
-        <f>IFERROR(VLOOKUP(C16,Pasted!$A$3:$AD$50,5,0),0)</f>
-        <v>18940</v>
+        <f>IFERROR(VLOOKUP(C16,Pasted!$A$3:$AD$50,7,0),0)</f>
+        <v>3252</v>
       </c>
       <c r="G16" s="1">
         <f>IFERROR(VLOOKUP(C16,Pasted!$A$3:$AD$50,9,0),0)</f>
@@ -7019,20 +7017,20 @@
         <v>329</v>
       </c>
       <c r="R16" s="1">
-        <f>IF(OR(VLOOKUP(C16,Pasted!$A$3:$AG$50,33,0)=1,LOWER(VLOOKUP(C16,Pasted!$A$3:$AG$50,33,0))="weekday"),1,0)</f>
+        <f>IF(OR(VLOOKUP(C16,Pasted!$A$3:$AI$50,35,0)=1,LOWER(VLOOKUP(C16,Pasted!$A$3:$AI$50,35,0))="weekday",LOWER(VLOOKUP(C16,Pasted!$A$3:$AI$50,35,0))="yes"),1,0)</f>
         <v>1</v>
       </c>
     </row>
     <row r="17" spans="1:18">
       <c r="A17" s="3" t="str">
-        <f>DAY(VLOOKUP(C17,Pasted!$A$3:$AF$50,32,0))&amp;" "&amp;CHOOSE(MONTH(VLOOKUP(C17,Pasted!$A$3:$AF$50,32,0)),"Jan","Feb","Mar","Apr","May","Jun","Jul","Aug","Sep","Oct","Nov","Dec")&amp;" "&amp;YEAR(VLOOKUP(C17,Pasted!$A$3:$AF$50,32,0))</f>
-        <v>29 May 2026</v>
+        <f>DAY(VLOOKUP(C17,Pasted!$A$3:$AH$50,34,0))&amp;" "&amp;CHOOSE(MONTH(VLOOKUP(C17,Pasted!$A$3:$AH$50,34,0)),"Jan","Feb","Mar","Apr","May","Jun","Jul","Aug","Sep","Oct","Nov","Dec")&amp;" "&amp;YEAR(VLOOKUP(C17,Pasted!$A$3:$AH$50,34,0))</f>
+        <v>12 May 2026</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="C17" s="1" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="D17" s="1">
         <v>1647</v>
@@ -7042,8 +7040,8 @@
         <v>33777</v>
       </c>
       <c r="F17" s="1">
-        <f>IFERROR(VLOOKUP(C17,Pasted!$A$3:$AD$50,5,0),0)</f>
-        <v>13745</v>
+        <f>IFERROR(VLOOKUP(C17,Pasted!$A$3:$AD$50,7,0),0)</f>
+        <v>4949</v>
       </c>
       <c r="G17" s="1">
         <f>IFERROR(VLOOKUP(C17,Pasted!$A$3:$AD$50,9,0),0)</f>
@@ -7089,14 +7087,14 @@
         <v>329</v>
       </c>
       <c r="R17" s="1">
-        <f>IF(OR(VLOOKUP(C17,Pasted!$A$3:$AG$50,33,0)=1,LOWER(VLOOKUP(C17,Pasted!$A$3:$AG$50,33,0))="weekday"),1,0)</f>
+        <f>IF(OR(VLOOKUP(C17,Pasted!$A$3:$AI$50,35,0)=1,LOWER(VLOOKUP(C17,Pasted!$A$3:$AI$50,35,0))="weekday",LOWER(VLOOKUP(C17,Pasted!$A$3:$AI$50,35,0))="yes"),1,0)</f>
         <v>1</v>
       </c>
     </row>
     <row r="18" spans="1:18">
       <c r="A18" s="3" t="str">
-        <f>DAY(VLOOKUP(C18,Pasted!$A$3:$AF$50,32,0))&amp;" "&amp;CHOOSE(MONTH(VLOOKUP(C18,Pasted!$A$3:$AF$50,32,0)),"Jan","Feb","Mar","Apr","May","Jun","Jul","Aug","Sep","Oct","Nov","Dec")&amp;" "&amp;YEAR(VLOOKUP(C18,Pasted!$A$3:$AF$50,32,0))</f>
-        <v>29 May 2026</v>
+        <f>DAY(VLOOKUP(C18,Pasted!$A$3:$AH$50,34,0))&amp;" "&amp;CHOOSE(MONTH(VLOOKUP(C18,Pasted!$A$3:$AH$50,34,0)),"Jan","Feb","Mar","Apr","May","Jun","Jul","Aug","Sep","Oct","Nov","Dec")&amp;" "&amp;YEAR(VLOOKUP(C18,Pasted!$A$3:$AH$50,34,0))</f>
+        <v>12 May 2026</v>
       </c>
       <c r="B18" s="1" t="s">
         <v>71</v>
@@ -7112,8 +7110,8 @@
         <v>34828</v>
       </c>
       <c r="F18" s="1">
-        <f>IFERROR(VLOOKUP(C18,Pasted!$A$3:$AD$50,5,0),0)</f>
-        <v>32964</v>
+        <f>IFERROR(VLOOKUP(C18,Pasted!$A$3:$AD$50,7,0),0)</f>
+        <v>305</v>
       </c>
       <c r="G18" s="1">
         <f>IFERROR(VLOOKUP(C18,Pasted!$A$3:$AD$50,9,0),0)</f>
@@ -7159,14 +7157,14 @@
         <v>329</v>
       </c>
       <c r="R18" s="1">
-        <f>IF(OR(VLOOKUP(C18,Pasted!$A$3:$AG$50,33,0)=1,LOWER(VLOOKUP(C18,Pasted!$A$3:$AG$50,33,0))="weekday"),1,0)</f>
+        <f>IF(OR(VLOOKUP(C18,Pasted!$A$3:$AI$50,35,0)=1,LOWER(VLOOKUP(C18,Pasted!$A$3:$AI$50,35,0))="weekday",LOWER(VLOOKUP(C18,Pasted!$A$3:$AI$50,35,0))="yes"),1,0)</f>
         <v>1</v>
       </c>
     </row>
     <row r="19" spans="1:18">
       <c r="A19" s="3" t="str">
-        <f>DAY(VLOOKUP(C19,Pasted!$A$3:$AF$50,32,0))&amp;" "&amp;CHOOSE(MONTH(VLOOKUP(C19,Pasted!$A$3:$AF$50,32,0)),"Jan","Feb","Mar","Apr","May","Jun","Jul","Aug","Sep","Oct","Nov","Dec")&amp;" "&amp;YEAR(VLOOKUP(C19,Pasted!$A$3:$AF$50,32,0))</f>
-        <v>29 May 2026</v>
+        <f>DAY(VLOOKUP(C19,Pasted!$A$3:$AH$50,34,0))&amp;" "&amp;CHOOSE(MONTH(VLOOKUP(C19,Pasted!$A$3:$AH$50,34,0)),"Jan","Feb","Mar","Apr","May","Jun","Jul","Aug","Sep","Oct","Nov","Dec")&amp;" "&amp;YEAR(VLOOKUP(C19,Pasted!$A$3:$AH$50,34,0))</f>
+        <v>12 May 2026</v>
       </c>
       <c r="B19" s="1" t="s">
         <v>20</v>
@@ -7182,8 +7180,8 @@
         <v>36969</v>
       </c>
       <c r="F19" s="1">
-        <f>IFERROR(VLOOKUP(C19,Pasted!$A$3:$AD$50,5,0),0)</f>
-        <v>36969</v>
+        <f>IFERROR(VLOOKUP(C19,Pasted!$A$3:$AD$50,7,0),0)</f>
+        <v>2</v>
       </c>
       <c r="G19" s="1">
         <f>IFERROR(VLOOKUP(C19,Pasted!$A$3:$AD$50,9,0),0)</f>
@@ -7229,20 +7227,20 @@
         <v>329</v>
       </c>
       <c r="R19" s="1">
-        <f>IF(OR(VLOOKUP(C19,Pasted!$A$3:$AG$50,33,0)=1,LOWER(VLOOKUP(C19,Pasted!$A$3:$AG$50,33,0))="weekday"),1,0)</f>
+        <f>IF(OR(VLOOKUP(C19,Pasted!$A$3:$AI$50,35,0)=1,LOWER(VLOOKUP(C19,Pasted!$A$3:$AI$50,35,0))="weekday",LOWER(VLOOKUP(C19,Pasted!$A$3:$AI$50,35,0))="yes"),1,0)</f>
         <v>1</v>
       </c>
     </row>
     <row r="20" spans="1:18">
       <c r="A20" s="3" t="str">
-        <f>DAY(VLOOKUP(C20,Pasted!$A$3:$AF$50,32,0))&amp;" "&amp;CHOOSE(MONTH(VLOOKUP(C20,Pasted!$A$3:$AF$50,32,0)),"Jan","Feb","Mar","Apr","May","Jun","Jul","Aug","Sep","Oct","Nov","Dec")&amp;" "&amp;YEAR(VLOOKUP(C20,Pasted!$A$3:$AF$50,32,0))</f>
-        <v>29 May 2026</v>
+        <f>DAY(VLOOKUP(C20,Pasted!$A$3:$AH$50,34,0))&amp;" "&amp;CHOOSE(MONTH(VLOOKUP(C20,Pasted!$A$3:$AH$50,34,0)),"Jan","Feb","Mar","Apr","May","Jun","Jul","Aug","Sep","Oct","Nov","Dec")&amp;" "&amp;YEAR(VLOOKUP(C20,Pasted!$A$3:$AH$50,34,0))</f>
+        <v>12 May 2026</v>
       </c>
       <c r="B20" s="1" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="C20" s="1" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="D20" s="1">
         <v>1651</v>
@@ -7252,8 +7250,8 @@
         <v>39176</v>
       </c>
       <c r="F20" s="1">
-        <f>IFERROR(VLOOKUP(C20,Pasted!$A$3:$AD$50,5,0),0)</f>
-        <v>20572</v>
+        <f>IFERROR(VLOOKUP(C20,Pasted!$A$3:$AD$50,7,0),0)</f>
+        <v>637</v>
       </c>
       <c r="G20" s="1">
         <f>IFERROR(VLOOKUP(C20,Pasted!$A$3:$AD$50,9,0),0)</f>
@@ -7299,14 +7297,14 @@
         <v>329</v>
       </c>
       <c r="R20" s="1">
-        <f>IF(OR(VLOOKUP(C20,Pasted!$A$3:$AG$50,33,0)=1,LOWER(VLOOKUP(C20,Pasted!$A$3:$AG$50,33,0))="weekday"),1,0)</f>
+        <f>IF(OR(VLOOKUP(C20,Pasted!$A$3:$AI$50,35,0)=1,LOWER(VLOOKUP(C20,Pasted!$A$3:$AI$50,35,0))="weekday",LOWER(VLOOKUP(C20,Pasted!$A$3:$AI$50,35,0))="yes"),1,0)</f>
         <v>1</v>
       </c>
     </row>
     <row r="21" spans="1:18">
       <c r="A21" s="3" t="str">
-        <f>DAY(VLOOKUP(C21,Pasted!$A$3:$AF$50,32,0))&amp;" "&amp;CHOOSE(MONTH(VLOOKUP(C21,Pasted!$A$3:$AF$50,32,0)),"Jan","Feb","Mar","Apr","May","Jun","Jul","Aug","Sep","Oct","Nov","Dec")&amp;" "&amp;YEAR(VLOOKUP(C21,Pasted!$A$3:$AF$50,32,0))</f>
-        <v>29 May 2026</v>
+        <f>DAY(VLOOKUP(C21,Pasted!$A$3:$AH$50,34,0))&amp;" "&amp;CHOOSE(MONTH(VLOOKUP(C21,Pasted!$A$3:$AH$50,34,0)),"Jan","Feb","Mar","Apr","May","Jun","Jul","Aug","Sep","Oct","Nov","Dec")&amp;" "&amp;YEAR(VLOOKUP(C21,Pasted!$A$3:$AH$50,34,0))</f>
+        <v>12 May 2026</v>
       </c>
       <c r="B21" s="1" t="s">
         <v>55</v>
@@ -7322,8 +7320,8 @@
         <v>36588</v>
       </c>
       <c r="F21" s="1">
-        <f>IFERROR(VLOOKUP(C21,Pasted!$A$3:$AD$50,5,0),0)</f>
-        <v>33154</v>
+        <f>IFERROR(VLOOKUP(C21,Pasted!$A$3:$AD$50,7,0),0)</f>
+        <v>172</v>
       </c>
       <c r="G21" s="1">
         <f>IFERROR(VLOOKUP(C21,Pasted!$A$3:$AD$50,9,0),0)</f>
@@ -7369,20 +7367,20 @@
         <v>329</v>
       </c>
       <c r="R21" s="1">
-        <f>IF(OR(VLOOKUP(C21,Pasted!$A$3:$AG$50,33,0)=1,LOWER(VLOOKUP(C21,Pasted!$A$3:$AG$50,33,0))="weekday"),1,0)</f>
+        <f>IF(OR(VLOOKUP(C21,Pasted!$A$3:$AI$50,35,0)=1,LOWER(VLOOKUP(C21,Pasted!$A$3:$AI$50,35,0))="weekday",LOWER(VLOOKUP(C21,Pasted!$A$3:$AI$50,35,0))="yes"),1,0)</f>
         <v>1</v>
       </c>
     </row>
     <row r="22" spans="1:18">
       <c r="A22" s="3" t="str">
-        <f>DAY(VLOOKUP(C22,Pasted!$A$3:$AF$50,32,0))&amp;" "&amp;CHOOSE(MONTH(VLOOKUP(C22,Pasted!$A$3:$AF$50,32,0)),"Jan","Feb","Mar","Apr","May","Jun","Jul","Aug","Sep","Oct","Nov","Dec")&amp;" "&amp;YEAR(VLOOKUP(C22,Pasted!$A$3:$AF$50,32,0))</f>
-        <v>29 May 2026</v>
+        <f>DAY(VLOOKUP(C22,Pasted!$A$3:$AH$50,34,0))&amp;" "&amp;CHOOSE(MONTH(VLOOKUP(C22,Pasted!$A$3:$AH$50,34,0)),"Jan","Feb","Mar","Apr","May","Jun","Jul","Aug","Sep","Oct","Nov","Dec")&amp;" "&amp;YEAR(VLOOKUP(C22,Pasted!$A$3:$AH$50,34,0))</f>
+        <v>12 May 2026</v>
       </c>
       <c r="B22" s="1" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="C22" s="1" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="D22" s="1">
         <v>1632</v>
@@ -7392,8 +7390,8 @@
         <v>39431</v>
       </c>
       <c r="F22" s="1">
-        <f>IFERROR(VLOOKUP(C22,Pasted!$A$3:$AD$50,5,0),0)</f>
-        <v>16851</v>
+        <f>IFERROR(VLOOKUP(C22,Pasted!$A$3:$AD$50,7,0),0)</f>
+        <v>1418</v>
       </c>
       <c r="G22" s="1">
         <f>IFERROR(VLOOKUP(C22,Pasted!$A$3:$AD$50,9,0),0)</f>
@@ -7439,20 +7437,20 @@
         <v>329</v>
       </c>
       <c r="R22" s="1">
-        <f>IF(OR(VLOOKUP(C22,Pasted!$A$3:$AG$50,33,0)=1,LOWER(VLOOKUP(C22,Pasted!$A$3:$AG$50,33,0))="weekday"),1,0)</f>
+        <f>IF(OR(VLOOKUP(C22,Pasted!$A$3:$AI$50,35,0)=1,LOWER(VLOOKUP(C22,Pasted!$A$3:$AI$50,35,0))="weekday",LOWER(VLOOKUP(C22,Pasted!$A$3:$AI$50,35,0))="yes"),1,0)</f>
         <v>1</v>
       </c>
     </row>
     <row r="23" spans="1:18">
       <c r="A23" s="3" t="str">
-        <f>DAY(VLOOKUP(C23,Pasted!$A$3:$AF$50,32,0))&amp;" "&amp;CHOOSE(MONTH(VLOOKUP(C23,Pasted!$A$3:$AF$50,32,0)),"Jan","Feb","Mar","Apr","May","Jun","Jul","Aug","Sep","Oct","Nov","Dec")&amp;" "&amp;YEAR(VLOOKUP(C23,Pasted!$A$3:$AF$50,32,0))</f>
-        <v>29 May 2026</v>
+        <f>DAY(VLOOKUP(C23,Pasted!$A$3:$AH$50,34,0))&amp;" "&amp;CHOOSE(MONTH(VLOOKUP(C23,Pasted!$A$3:$AH$50,34,0)),"Jan","Feb","Mar","Apr","May","Jun","Jul","Aug","Sep","Oct","Nov","Dec")&amp;" "&amp;YEAR(VLOOKUP(C23,Pasted!$A$3:$AH$50,34,0))</f>
+        <v>12 May 2026</v>
       </c>
       <c r="B23" s="1" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="C23" s="1" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="D23" s="1">
         <v>1616</v>
@@ -7462,7 +7460,7 @@
         <v>9</v>
       </c>
       <c r="F23" s="1">
-        <f>IFERROR(VLOOKUP(C23,Pasted!$A$3:$AD$50,5,0),0)</f>
+        <f>IFERROR(VLOOKUP(C23,Pasted!$A$3:$AD$50,7,0),0)</f>
         <v>9</v>
       </c>
       <c r="G23" s="1">
@@ -7509,14 +7507,14 @@
         <v>329</v>
       </c>
       <c r="R23" s="1">
-        <f>IF(OR(VLOOKUP(C23,Pasted!$A$3:$AG$50,33,0)=1,LOWER(VLOOKUP(C23,Pasted!$A$3:$AG$50,33,0))="weekday"),1,0)</f>
+        <f>IF(OR(VLOOKUP(C23,Pasted!$A$3:$AI$50,35,0)=1,LOWER(VLOOKUP(C23,Pasted!$A$3:$AI$50,35,0))="weekday",LOWER(VLOOKUP(C23,Pasted!$A$3:$AI$50,35,0))="yes"),1,0)</f>
         <v>1</v>
       </c>
     </row>
     <row r="24" spans="1:18">
       <c r="A24" s="3" t="str">
-        <f>DAY(VLOOKUP(C24,Pasted!$A$3:$AF$50,32,0))&amp;" "&amp;CHOOSE(MONTH(VLOOKUP(C24,Pasted!$A$3:$AF$50,32,0)),"Jan","Feb","Mar","Apr","May","Jun","Jul","Aug","Sep","Oct","Nov","Dec")&amp;" "&amp;YEAR(VLOOKUP(C24,Pasted!$A$3:$AF$50,32,0))</f>
-        <v>29 May 2026</v>
+        <f>DAY(VLOOKUP(C24,Pasted!$A$3:$AH$50,34,0))&amp;" "&amp;CHOOSE(MONTH(VLOOKUP(C24,Pasted!$A$3:$AH$50,34,0)),"Jan","Feb","Mar","Apr","May","Jun","Jul","Aug","Sep","Oct","Nov","Dec")&amp;" "&amp;YEAR(VLOOKUP(C24,Pasted!$A$3:$AH$50,34,0))</f>
+        <v>12 May 2026</v>
       </c>
       <c r="B24" s="1" t="s">
         <v>113</v>
@@ -7532,8 +7530,8 @@
         <v>34419</v>
       </c>
       <c r="F24" s="1">
-        <f>IFERROR(VLOOKUP(C24,Pasted!$A$3:$AD$50,5,0),0)</f>
-        <v>26285</v>
+        <f>IFERROR(VLOOKUP(C24,Pasted!$A$3:$AD$50,7,0),0)</f>
+        <v>3679</v>
       </c>
       <c r="G24" s="1">
         <f>IFERROR(VLOOKUP(C24,Pasted!$A$3:$AD$50,9,0),0)</f>
@@ -7579,20 +7577,20 @@
         <v>329</v>
       </c>
       <c r="R24" s="1">
-        <f>IF(OR(VLOOKUP(C24,Pasted!$A$3:$AG$50,33,0)=1,LOWER(VLOOKUP(C24,Pasted!$A$3:$AG$50,33,0))="weekday"),1,0)</f>
+        <f>IF(OR(VLOOKUP(C24,Pasted!$A$3:$AI$50,35,0)=1,LOWER(VLOOKUP(C24,Pasted!$A$3:$AI$50,35,0))="weekday",LOWER(VLOOKUP(C24,Pasted!$A$3:$AI$50,35,0))="yes"),1,0)</f>
         <v>1</v>
       </c>
     </row>
     <row r="25" spans="1:18">
       <c r="A25" s="3" t="str">
-        <f>DAY(VLOOKUP(C25,Pasted!$A$3:$AF$50,32,0))&amp;" "&amp;CHOOSE(MONTH(VLOOKUP(C25,Pasted!$A$3:$AF$50,32,0)),"Jan","Feb","Mar","Apr","May","Jun","Jul","Aug","Sep","Oct","Nov","Dec")&amp;" "&amp;YEAR(VLOOKUP(C25,Pasted!$A$3:$AF$50,32,0))</f>
-        <v>29 May 2026</v>
+        <f>DAY(VLOOKUP(C25,Pasted!$A$3:$AH$50,34,0))&amp;" "&amp;CHOOSE(MONTH(VLOOKUP(C25,Pasted!$A$3:$AH$50,34,0)),"Jan","Feb","Mar","Apr","May","Jun","Jul","Aug","Sep","Oct","Nov","Dec")&amp;" "&amp;YEAR(VLOOKUP(C25,Pasted!$A$3:$AH$50,34,0))</f>
+        <v>12 May 2026</v>
       </c>
       <c r="B25" s="1" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="C25" s="1" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="D25" s="1">
         <v>1630</v>
@@ -7602,8 +7600,8 @@
         <v>35712</v>
       </c>
       <c r="F25" s="1">
-        <f>IFERROR(VLOOKUP(C25,Pasted!$A$3:$AD$50,5,0),0)</f>
-        <v>16882</v>
+        <f>IFERROR(VLOOKUP(C25,Pasted!$A$3:$AD$50,7,0),0)</f>
+        <v>1998</v>
       </c>
       <c r="G25" s="1">
         <f>IFERROR(VLOOKUP(C25,Pasted!$A$3:$AD$50,9,0),0)</f>
@@ -7649,14 +7647,14 @@
         <v>329</v>
       </c>
       <c r="R25" s="1">
-        <f>IF(OR(VLOOKUP(C25,Pasted!$A$3:$AG$50,33,0)=1,LOWER(VLOOKUP(C25,Pasted!$A$3:$AG$50,33,0))="weekday"),1,0)</f>
+        <f>IF(OR(VLOOKUP(C25,Pasted!$A$3:$AI$50,35,0)=1,LOWER(VLOOKUP(C25,Pasted!$A$3:$AI$50,35,0))="weekday",LOWER(VLOOKUP(C25,Pasted!$A$3:$AI$50,35,0))="yes"),1,0)</f>
         <v>1</v>
       </c>
     </row>
     <row r="26" spans="1:18">
       <c r="A26" s="3" t="str">
-        <f>DAY(VLOOKUP(C26,Pasted!$A$3:$AF$50,32,0))&amp;" "&amp;CHOOSE(MONTH(VLOOKUP(C26,Pasted!$A$3:$AF$50,32,0)),"Jan","Feb","Mar","Apr","May","Jun","Jul","Aug","Sep","Oct","Nov","Dec")&amp;" "&amp;YEAR(VLOOKUP(C26,Pasted!$A$3:$AF$50,32,0))</f>
-        <v>29 May 2026</v>
+        <f>DAY(VLOOKUP(C26,Pasted!$A$3:$AH$50,34,0))&amp;" "&amp;CHOOSE(MONTH(VLOOKUP(C26,Pasted!$A$3:$AH$50,34,0)),"Jan","Feb","Mar","Apr","May","Jun","Jul","Aug","Sep","Oct","Nov","Dec")&amp;" "&amp;YEAR(VLOOKUP(C26,Pasted!$A$3:$AH$50,34,0))</f>
+        <v>12 May 2026</v>
       </c>
       <c r="B26" s="1" t="s">
         <v>47</v>
@@ -7672,8 +7670,8 @@
         <v>33788</v>
       </c>
       <c r="F26" s="1">
-        <f>IFERROR(VLOOKUP(C26,Pasted!$A$3:$AD$50,5,0),0)</f>
-        <v>33788</v>
+        <f>IFERROR(VLOOKUP(C26,Pasted!$A$3:$AD$50,7,0),0)</f>
+        <v>3</v>
       </c>
       <c r="G26" s="1">
         <f>IFERROR(VLOOKUP(C26,Pasted!$A$3:$AD$50,9,0),0)</f>
@@ -7719,20 +7717,20 @@
         <v>329</v>
       </c>
       <c r="R26" s="1">
-        <f>IF(OR(VLOOKUP(C26,Pasted!$A$3:$AG$50,33,0)=1,LOWER(VLOOKUP(C26,Pasted!$A$3:$AG$50,33,0))="weekday"),1,0)</f>
+        <f>IF(OR(VLOOKUP(C26,Pasted!$A$3:$AI$50,35,0)=1,LOWER(VLOOKUP(C26,Pasted!$A$3:$AI$50,35,0))="weekday",LOWER(VLOOKUP(C26,Pasted!$A$3:$AI$50,35,0))="yes"),1,0)</f>
         <v>1</v>
       </c>
     </row>
     <row r="27" spans="1:18">
       <c r="A27" s="3" t="str">
-        <f>DAY(VLOOKUP(C27,Pasted!$A$3:$AF$50,32,0))&amp;" "&amp;CHOOSE(MONTH(VLOOKUP(C27,Pasted!$A$3:$AF$50,32,0)),"Jan","Feb","Mar","Apr","May","Jun","Jul","Aug","Sep","Oct","Nov","Dec")&amp;" "&amp;YEAR(VLOOKUP(C27,Pasted!$A$3:$AF$50,32,0))</f>
-        <v>29 May 2026</v>
+        <f>DAY(VLOOKUP(C27,Pasted!$A$3:$AH$50,34,0))&amp;" "&amp;CHOOSE(MONTH(VLOOKUP(C27,Pasted!$A$3:$AH$50,34,0)),"Jan","Feb","Mar","Apr","May","Jun","Jul","Aug","Sep","Oct","Nov","Dec")&amp;" "&amp;YEAR(VLOOKUP(C27,Pasted!$A$3:$AH$50,34,0))</f>
+        <v>12 May 2026</v>
       </c>
       <c r="B27" s="1" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="C27" s="1" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="D27" s="1">
         <v>1653</v>
@@ -7742,8 +7740,8 @@
         <v>39232</v>
       </c>
       <c r="F27" s="1">
-        <f>IFERROR(VLOOKUP(C27,Pasted!$A$3:$AD$50,5,0),0)</f>
-        <v>17403</v>
+        <f>IFERROR(VLOOKUP(C27,Pasted!$A$3:$AD$50,7,0),0)</f>
+        <v>363</v>
       </c>
       <c r="G27" s="1">
         <f>IFERROR(VLOOKUP(C27,Pasted!$A$3:$AD$50,9,0),0)</f>
@@ -7789,14 +7787,14 @@
         <v>329</v>
       </c>
       <c r="R27" s="1">
-        <f>IF(OR(VLOOKUP(C27,Pasted!$A$3:$AG$50,33,0)=1,LOWER(VLOOKUP(C27,Pasted!$A$3:$AG$50,33,0))="weekday"),1,0)</f>
+        <f>IF(OR(VLOOKUP(C27,Pasted!$A$3:$AI$50,35,0)=1,LOWER(VLOOKUP(C27,Pasted!$A$3:$AI$50,35,0))="weekday",LOWER(VLOOKUP(C27,Pasted!$A$3:$AI$50,35,0))="yes"),1,0)</f>
         <v>1</v>
       </c>
     </row>
     <row r="28" spans="1:18">
       <c r="A28" s="3" t="str">
-        <f>DAY(VLOOKUP(C28,Pasted!$A$3:$AF$50,32,0))&amp;" "&amp;CHOOSE(MONTH(VLOOKUP(C28,Pasted!$A$3:$AF$50,32,0)),"Jan","Feb","Mar","Apr","May","Jun","Jul","Aug","Sep","Oct","Nov","Dec")&amp;" "&amp;YEAR(VLOOKUP(C28,Pasted!$A$3:$AF$50,32,0))</f>
-        <v>29 May 2026</v>
+        <f>DAY(VLOOKUP(C28,Pasted!$A$3:$AH$50,34,0))&amp;" "&amp;CHOOSE(MONTH(VLOOKUP(C28,Pasted!$A$3:$AH$50,34,0)),"Jan","Feb","Mar","Apr","May","Jun","Jul","Aug","Sep","Oct","Nov","Dec")&amp;" "&amp;YEAR(VLOOKUP(C28,Pasted!$A$3:$AH$50,34,0))</f>
+        <v>12 May 2026</v>
       </c>
       <c r="B28" s="1" t="s">
         <v>147</v>
@@ -7812,8 +7810,8 @@
         <v>34718</v>
       </c>
       <c r="F28" s="1">
-        <f>IFERROR(VLOOKUP(C28,Pasted!$A$3:$AD$50,5,0),0)</f>
-        <v>21467</v>
+        <f>IFERROR(VLOOKUP(C28,Pasted!$A$3:$AD$50,7,0),0)</f>
+        <v>896</v>
       </c>
       <c r="G28" s="1">
         <f>IFERROR(VLOOKUP(C28,Pasted!$A$3:$AD$50,9,0),0)</f>
@@ -7859,14 +7857,14 @@
         <v>329</v>
       </c>
       <c r="R28" s="1">
-        <f>IF(OR(VLOOKUP(C28,Pasted!$A$3:$AG$50,33,0)=1,LOWER(VLOOKUP(C28,Pasted!$A$3:$AG$50,33,0))="weekday"),1,0)</f>
+        <f>IF(OR(VLOOKUP(C28,Pasted!$A$3:$AI$50,35,0)=1,LOWER(VLOOKUP(C28,Pasted!$A$3:$AI$50,35,0))="weekday",LOWER(VLOOKUP(C28,Pasted!$A$3:$AI$50,35,0))="yes"),1,0)</f>
         <v>1</v>
       </c>
     </row>
     <row r="29" spans="1:18">
       <c r="A29" s="3" t="str">
-        <f>DAY(VLOOKUP(C29,Pasted!$A$3:$AF$50,32,0))&amp;" "&amp;CHOOSE(MONTH(VLOOKUP(C29,Pasted!$A$3:$AF$50,32,0)),"Jan","Feb","Mar","Apr","May","Jun","Jul","Aug","Sep","Oct","Nov","Dec")&amp;" "&amp;YEAR(VLOOKUP(C29,Pasted!$A$3:$AF$50,32,0))</f>
-        <v>29 May 2026</v>
+        <f>DAY(VLOOKUP(C29,Pasted!$A$3:$AH$50,34,0))&amp;" "&amp;CHOOSE(MONTH(VLOOKUP(C29,Pasted!$A$3:$AH$50,34,0)),"Jan","Feb","Mar","Apr","May","Jun","Jul","Aug","Sep","Oct","Nov","Dec")&amp;" "&amp;YEAR(VLOOKUP(C29,Pasted!$A$3:$AH$50,34,0))</f>
+        <v>12 May 2026</v>
       </c>
       <c r="B29" s="1" t="s">
         <v>27</v>
@@ -7882,8 +7880,8 @@
         <v>34799</v>
       </c>
       <c r="F29" s="1">
-        <f>IFERROR(VLOOKUP(C29,Pasted!$A$3:$AD$50,5,0),0)</f>
-        <v>34799</v>
+        <f>IFERROR(VLOOKUP(C29,Pasted!$A$3:$AD$50,7,0),0)</f>
+        <v>5</v>
       </c>
       <c r="G29" s="1">
         <f>IFERROR(VLOOKUP(C29,Pasted!$A$3:$AD$50,9,0),0)</f>
@@ -7929,14 +7927,14 @@
         <v>329</v>
       </c>
       <c r="R29" s="1">
-        <f>IF(OR(VLOOKUP(C29,Pasted!$A$3:$AG$50,33,0)=1,LOWER(VLOOKUP(C29,Pasted!$A$3:$AG$50,33,0))="weekday"),1,0)</f>
+        <f>IF(OR(VLOOKUP(C29,Pasted!$A$3:$AI$50,35,0)=1,LOWER(VLOOKUP(C29,Pasted!$A$3:$AI$50,35,0))="weekday",LOWER(VLOOKUP(C29,Pasted!$A$3:$AI$50,35,0))="yes"),1,0)</f>
         <v>1</v>
       </c>
     </row>
     <row r="30" spans="1:18">
       <c r="A30" s="3" t="str">
-        <f>DAY(VLOOKUP(C30,Pasted!$A$3:$AF$50,32,0))&amp;" "&amp;CHOOSE(MONTH(VLOOKUP(C30,Pasted!$A$3:$AF$50,32,0)),"Jan","Feb","Mar","Apr","May","Jun","Jul","Aug","Sep","Oct","Nov","Dec")&amp;" "&amp;YEAR(VLOOKUP(C30,Pasted!$A$3:$AF$50,32,0))</f>
-        <v>29 May 2026</v>
+        <f>DAY(VLOOKUP(C30,Pasted!$A$3:$AH$50,34,0))&amp;" "&amp;CHOOSE(MONTH(VLOOKUP(C30,Pasted!$A$3:$AH$50,34,0)),"Jan","Feb","Mar","Apr","May","Jun","Jul","Aug","Sep","Oct","Nov","Dec")&amp;" "&amp;YEAR(VLOOKUP(C30,Pasted!$A$3:$AH$50,34,0))</f>
+        <v>12 May 2026</v>
       </c>
       <c r="B30" s="1" t="s">
         <v>92</v>
@@ -7952,8 +7950,8 @@
         <v>35571</v>
       </c>
       <c r="F30" s="1">
-        <f>IFERROR(VLOOKUP(C30,Pasted!$A$3:$AD$50,5,0),0)</f>
-        <v>28350</v>
+        <f>IFERROR(VLOOKUP(C30,Pasted!$A$3:$AD$50,7,0),0)</f>
+        <v>1780</v>
       </c>
       <c r="G30" s="1">
         <f>IFERROR(VLOOKUP(C30,Pasted!$A$3:$AD$50,9,0),0)</f>
@@ -7999,20 +7997,20 @@
         <v>329</v>
       </c>
       <c r="R30" s="1">
-        <f>IF(OR(VLOOKUP(C30,Pasted!$A$3:$AG$50,33,0)=1,LOWER(VLOOKUP(C30,Pasted!$A$3:$AG$50,33,0))="weekday"),1,0)</f>
+        <f>IF(OR(VLOOKUP(C30,Pasted!$A$3:$AI$50,35,0)=1,LOWER(VLOOKUP(C30,Pasted!$A$3:$AI$50,35,0))="weekday",LOWER(VLOOKUP(C30,Pasted!$A$3:$AI$50,35,0))="yes"),1,0)</f>
         <v>1</v>
       </c>
     </row>
     <row r="31" spans="1:18">
       <c r="A31" s="3" t="str">
-        <f>DAY(VLOOKUP(C31,Pasted!$A$3:$AF$50,32,0))&amp;" "&amp;CHOOSE(MONTH(VLOOKUP(C31,Pasted!$A$3:$AF$50,32,0)),"Jan","Feb","Mar","Apr","May","Jun","Jul","Aug","Sep","Oct","Nov","Dec")&amp;" "&amp;YEAR(VLOOKUP(C31,Pasted!$A$3:$AF$50,32,0))</f>
-        <v>29 May 2026</v>
+        <f>DAY(VLOOKUP(C31,Pasted!$A$3:$AH$50,34,0))&amp;" "&amp;CHOOSE(MONTH(VLOOKUP(C31,Pasted!$A$3:$AH$50,34,0)),"Jan","Feb","Mar","Apr","May","Jun","Jul","Aug","Sep","Oct","Nov","Dec")&amp;" "&amp;YEAR(VLOOKUP(C31,Pasted!$A$3:$AH$50,34,0))</f>
+        <v>12 May 2026</v>
       </c>
       <c r="B31" s="1" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="C31" s="1" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="D31" s="1">
         <v>1641</v>
@@ -8022,8 +8020,8 @@
         <v>35631</v>
       </c>
       <c r="F31" s="1">
-        <f>IFERROR(VLOOKUP(C31,Pasted!$A$3:$AD$50,5,0),0)</f>
-        <v>16429</v>
+        <f>IFERROR(VLOOKUP(C31,Pasted!$A$3:$AD$50,7,0),0)</f>
+        <v>2331</v>
       </c>
       <c r="G31" s="1">
         <f>IFERROR(VLOOKUP(C31,Pasted!$A$3:$AD$50,9,0),0)</f>
@@ -8069,14 +8067,14 @@
         <v>329</v>
       </c>
       <c r="R31" s="1">
-        <f>IF(OR(VLOOKUP(C31,Pasted!$A$3:$AG$50,33,0)=1,LOWER(VLOOKUP(C31,Pasted!$A$3:$AG$50,33,0))="weekday"),1,0)</f>
+        <f>IF(OR(VLOOKUP(C31,Pasted!$A$3:$AI$50,35,0)=1,LOWER(VLOOKUP(C31,Pasted!$A$3:$AI$50,35,0))="weekday",LOWER(VLOOKUP(C31,Pasted!$A$3:$AI$50,35,0))="yes"),1,0)</f>
         <v>1</v>
       </c>
     </row>
     <row r="32" spans="1:18">
       <c r="A32" s="3" t="str">
-        <f>DAY(VLOOKUP(C32,Pasted!$A$3:$AF$50,32,0))&amp;" "&amp;CHOOSE(MONTH(VLOOKUP(C32,Pasted!$A$3:$AF$50,32,0)),"Jan","Feb","Mar","Apr","May","Jun","Jul","Aug","Sep","Oct","Nov","Dec")&amp;" "&amp;YEAR(VLOOKUP(C32,Pasted!$A$3:$AF$50,32,0))</f>
-        <v>29 May 2026</v>
+        <f>DAY(VLOOKUP(C32,Pasted!$A$3:$AH$50,34,0))&amp;" "&amp;CHOOSE(MONTH(VLOOKUP(C32,Pasted!$A$3:$AH$50,34,0)),"Jan","Feb","Mar","Apr","May","Jun","Jul","Aug","Sep","Oct","Nov","Dec")&amp;" "&amp;YEAR(VLOOKUP(C32,Pasted!$A$3:$AH$50,34,0))</f>
+        <v>12 May 2026</v>
       </c>
       <c r="B32" s="1" t="s">
         <v>131</v>
@@ -8092,8 +8090,8 @@
         <v>33536</v>
       </c>
       <c r="F32" s="1">
-        <f>IFERROR(VLOOKUP(C32,Pasted!$A$3:$AD$50,5,0),0)</f>
-        <v>21995</v>
+        <f>IFERROR(VLOOKUP(C32,Pasted!$A$3:$AD$50,7,0),0)</f>
+        <v>3654</v>
       </c>
       <c r="G32" s="1">
         <f>IFERROR(VLOOKUP(C32,Pasted!$A$3:$AD$50,9,0),0)</f>
@@ -8139,14 +8137,14 @@
         <v>329</v>
       </c>
       <c r="R32" s="1">
-        <f>IF(OR(VLOOKUP(C32,Pasted!$A$3:$AG$50,33,0)=1,LOWER(VLOOKUP(C32,Pasted!$A$3:$AG$50,33,0))="weekday"),1,0)</f>
+        <f>IF(OR(VLOOKUP(C32,Pasted!$A$3:$AI$50,35,0)=1,LOWER(VLOOKUP(C32,Pasted!$A$3:$AI$50,35,0))="weekday",LOWER(VLOOKUP(C32,Pasted!$A$3:$AI$50,35,0))="yes"),1,0)</f>
         <v>1</v>
       </c>
     </row>
     <row r="33" spans="1:18">
       <c r="A33" s="3" t="str">
-        <f>DAY(VLOOKUP(C33,Pasted!$A$3:$AF$50,32,0))&amp;" "&amp;CHOOSE(MONTH(VLOOKUP(C33,Pasted!$A$3:$AF$50,32,0)),"Jan","Feb","Mar","Apr","May","Jun","Jul","Aug","Sep","Oct","Nov","Dec")&amp;" "&amp;YEAR(VLOOKUP(C33,Pasted!$A$3:$AF$50,32,0))</f>
-        <v>29 May 2026</v>
+        <f>DAY(VLOOKUP(C33,Pasted!$A$3:$AH$50,34,0))&amp;" "&amp;CHOOSE(MONTH(VLOOKUP(C33,Pasted!$A$3:$AH$50,34,0)),"Jan","Feb","Mar","Apr","May","Jun","Jul","Aug","Sep","Oct","Nov","Dec")&amp;" "&amp;YEAR(VLOOKUP(C33,Pasted!$A$3:$AH$50,34,0))</f>
+        <v>12 May 2026</v>
       </c>
       <c r="B33" s="1" t="s">
         <v>122</v>
@@ -8162,8 +8160,8 @@
         <v>35051</v>
       </c>
       <c r="F33" s="1">
-        <f>IFERROR(VLOOKUP(C33,Pasted!$A$3:$AD$50,5,0),0)</f>
-        <v>23785</v>
+        <f>IFERROR(VLOOKUP(C33,Pasted!$A$3:$AD$50,7,0),0)</f>
+        <v>1913</v>
       </c>
       <c r="G33" s="1">
         <f>IFERROR(VLOOKUP(C33,Pasted!$A$3:$AD$50,9,0),0)</f>
@@ -8209,14 +8207,14 @@
         <v>329</v>
       </c>
       <c r="R33" s="1">
-        <f>IF(OR(VLOOKUP(C33,Pasted!$A$3:$AG$50,33,0)=1,LOWER(VLOOKUP(C33,Pasted!$A$3:$AG$50,33,0))="weekday"),1,0)</f>
+        <f>IF(OR(VLOOKUP(C33,Pasted!$A$3:$AI$50,35,0)=1,LOWER(VLOOKUP(C33,Pasted!$A$3:$AI$50,35,0))="weekday",LOWER(VLOOKUP(C33,Pasted!$A$3:$AI$50,35,0))="yes"),1,0)</f>
         <v>1</v>
       </c>
     </row>
     <row r="34" spans="1:18">
       <c r="A34" s="3" t="str">
-        <f>DAY(VLOOKUP(C34,Pasted!$A$3:$AF$50,32,0))&amp;" "&amp;CHOOSE(MONTH(VLOOKUP(C34,Pasted!$A$3:$AF$50,32,0)),"Jan","Feb","Mar","Apr","May","Jun","Jul","Aug","Sep","Oct","Nov","Dec")&amp;" "&amp;YEAR(VLOOKUP(C34,Pasted!$A$3:$AF$50,32,0))</f>
-        <v>29 May 2026</v>
+        <f>DAY(VLOOKUP(C34,Pasted!$A$3:$AH$50,34,0))&amp;" "&amp;CHOOSE(MONTH(VLOOKUP(C34,Pasted!$A$3:$AH$50,34,0)),"Jan","Feb","Mar","Apr","May","Jun","Jul","Aug","Sep","Oct","Nov","Dec")&amp;" "&amp;YEAR(VLOOKUP(C34,Pasted!$A$3:$AH$50,34,0))</f>
+        <v>12 May 2026</v>
       </c>
       <c r="B34" s="1" t="s">
         <v>34</v>
@@ -8232,8 +8230,8 @@
         <v>34785</v>
       </c>
       <c r="F34" s="1">
-        <f>IFERROR(VLOOKUP(C34,Pasted!$A$3:$AD$50,5,0),0)</f>
-        <v>34785</v>
+        <f>IFERROR(VLOOKUP(C34,Pasted!$A$3:$AD$50,7,0),0)</f>
+        <v>2913</v>
       </c>
       <c r="G34" s="1">
         <f>IFERROR(VLOOKUP(C34,Pasted!$A$3:$AD$50,9,0),0)</f>
@@ -8279,20 +8277,20 @@
         <v>329</v>
       </c>
       <c r="R34" s="1">
-        <f>IF(OR(VLOOKUP(C34,Pasted!$A$3:$AG$50,33,0)=1,LOWER(VLOOKUP(C34,Pasted!$A$3:$AG$50,33,0))="weekday"),1,0)</f>
+        <f>IF(OR(VLOOKUP(C34,Pasted!$A$3:$AI$50,35,0)=1,LOWER(VLOOKUP(C34,Pasted!$A$3:$AI$50,35,0))="weekday",LOWER(VLOOKUP(C34,Pasted!$A$3:$AI$50,35,0))="yes"),1,0)</f>
         <v>1</v>
       </c>
     </row>
     <row r="35" spans="1:18">
       <c r="A35" s="3" t="str">
-        <f>DAY(VLOOKUP(C35,Pasted!$A$3:$AF$50,32,0))&amp;" "&amp;CHOOSE(MONTH(VLOOKUP(C35,Pasted!$A$3:$AF$50,32,0)),"Jan","Feb","Mar","Apr","May","Jun","Jul","Aug","Sep","Oct","Nov","Dec")&amp;" "&amp;YEAR(VLOOKUP(C35,Pasted!$A$3:$AF$50,32,0))</f>
-        <v>29 May 2026</v>
+        <f>DAY(VLOOKUP(C35,Pasted!$A$3:$AH$50,34,0))&amp;" "&amp;CHOOSE(MONTH(VLOOKUP(C35,Pasted!$A$3:$AH$50,34,0)),"Jan","Feb","Mar","Apr","May","Jun","Jul","Aug","Sep","Oct","Nov","Dec")&amp;" "&amp;YEAR(VLOOKUP(C35,Pasted!$A$3:$AH$50,34,0))</f>
+        <v>12 May 2026</v>
       </c>
       <c r="B35" s="1" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
       <c r="C35" s="1" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
       <c r="D35" s="1">
         <v>1621</v>
@@ -8302,8 +8300,8 @@
         <v>36238</v>
       </c>
       <c r="F35" s="1">
-        <f>IFERROR(VLOOKUP(C35,Pasted!$A$3:$AD$50,5,0),0)</f>
-        <v>13343</v>
+        <f>IFERROR(VLOOKUP(C35,Pasted!$A$3:$AD$50,7,0),0)</f>
+        <v>3461</v>
       </c>
       <c r="G35" s="1">
         <f>IFERROR(VLOOKUP(C35,Pasted!$A$3:$AD$50,9,0),0)</f>
@@ -8349,7 +8347,7 @@
         <v>329</v>
       </c>
       <c r="R35" s="1">
-        <f>IF(OR(VLOOKUP(C35,Pasted!$A$3:$AG$50,33,0)=1,LOWER(VLOOKUP(C35,Pasted!$A$3:$AG$50,33,0))="weekday"),1,0)</f>
+        <f>IF(OR(VLOOKUP(C35,Pasted!$A$3:$AI$50,35,0)=1,LOWER(VLOOKUP(C35,Pasted!$A$3:$AI$50,35,0))="weekday",LOWER(VLOOKUP(C35,Pasted!$A$3:$AI$50,35,0))="yes"),1,0)</f>
         <v>1</v>
       </c>
     </row>

</xml_diff>